<commit_message>
Nightly oil data update
</commit_message>
<xml_diff>
--- a/oil_collection_report.xlsx
+++ b/oil_collection_report.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DX140"/>
+  <dimension ref="A1:DW140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1079,11 +1079,6 @@
       </c>
       <c r="DW1" t="inlineStr">
         <is>
-          <t>Worcester</t>
-        </is>
-      </c>
-      <c r="DX1" t="inlineStr">
-        <is>
           <t>ROW_TOTAL</t>
         </is>
       </c>
@@ -1470,9 +1465,6 @@
         <v>105</v>
       </c>
       <c r="DW2" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX2" t="n">
         <v>3913</v>
       </c>
     </row>
@@ -1858,9 +1850,6 @@
         <v>0</v>
       </c>
       <c r="DW3" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX3" t="n">
         <v>3042</v>
       </c>
     </row>
@@ -2246,9 +2235,6 @@
         <v>90</v>
       </c>
       <c r="DW4" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX4" t="n">
         <v>3428</v>
       </c>
     </row>
@@ -2634,9 +2620,6 @@
         <v>145</v>
       </c>
       <c r="DW5" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX5" t="n">
         <v>6856</v>
       </c>
     </row>
@@ -3022,9 +3005,6 @@
         <v>80</v>
       </c>
       <c r="DW6" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX6" t="n">
         <v>4864</v>
       </c>
     </row>
@@ -3083,7 +3063,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>1581</v>
+        <v>1606</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
@@ -3410,9 +3390,6 @@
         <v>120</v>
       </c>
       <c r="DW7" t="n">
-        <v>25</v>
-      </c>
-      <c r="DX7" t="n">
         <v>4418</v>
       </c>
     </row>
@@ -3798,9 +3775,6 @@
         <v>105</v>
       </c>
       <c r="DW8" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX8" t="n">
         <v>4482</v>
       </c>
     </row>
@@ -4186,9 +4160,6 @@
         <v>0</v>
       </c>
       <c r="DW9" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX9" t="n">
         <v>5047</v>
       </c>
     </row>
@@ -4574,9 +4545,6 @@
         <v>170</v>
       </c>
       <c r="DW10" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX10" t="n">
         <v>5877</v>
       </c>
     </row>
@@ -4962,9 +4930,6 @@
         <v>95</v>
       </c>
       <c r="DW11" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX11" t="n">
         <v>4120</v>
       </c>
     </row>
@@ -5350,9 +5315,6 @@
         <v>112</v>
       </c>
       <c r="DW12" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX12" t="n">
         <v>5336</v>
       </c>
     </row>
@@ -5411,7 +5373,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>2077</v>
+        <v>2092</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
@@ -5738,9 +5700,6 @@
         <v>60</v>
       </c>
       <c r="DW13" t="n">
-        <v>15</v>
-      </c>
-      <c r="DX13" t="n">
         <v>5301</v>
       </c>
     </row>
@@ -6126,9 +6085,6 @@
         <v>145</v>
       </c>
       <c r="DW14" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX14" t="n">
         <v>4432</v>
       </c>
     </row>
@@ -6514,9 +6470,6 @@
         <v>80</v>
       </c>
       <c r="DW15" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX15" t="n">
         <v>6308</v>
       </c>
     </row>
@@ -6902,9 +6855,6 @@
         <v>200</v>
       </c>
       <c r="DW16" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX16" t="n">
         <v>5676</v>
       </c>
     </row>
@@ -7290,9 +7240,6 @@
         <v>100</v>
       </c>
       <c r="DW17" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX17" t="n">
         <v>6593</v>
       </c>
     </row>
@@ -7678,9 +7625,6 @@
         <v>0</v>
       </c>
       <c r="DW18" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX18" t="n">
         <v>7082</v>
       </c>
     </row>
@@ -8066,9 +8010,6 @@
         <v>265</v>
       </c>
       <c r="DW19" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX19" t="n">
         <v>10586</v>
       </c>
     </row>
@@ -8454,9 +8395,6 @@
         <v>80</v>
       </c>
       <c r="DW20" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX20" t="n">
         <v>13147</v>
       </c>
     </row>
@@ -8842,9 +8780,6 @@
         <v>110</v>
       </c>
       <c r="DW21" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX21" t="n">
         <v>7916</v>
       </c>
     </row>
@@ -9230,9 +9165,6 @@
         <v>265</v>
       </c>
       <c r="DW22" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX22" t="n">
         <v>8012</v>
       </c>
     </row>
@@ -9618,9 +9550,6 @@
         <v>175</v>
       </c>
       <c r="DW23" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX23" t="n">
         <v>8118</v>
       </c>
     </row>
@@ -10006,9 +9935,6 @@
         <v>155</v>
       </c>
       <c r="DW24" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX24" t="n">
         <v>6385</v>
       </c>
     </row>
@@ -10394,9 +10320,6 @@
         <v>100</v>
       </c>
       <c r="DW25" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX25" t="n">
         <v>6113</v>
       </c>
     </row>
@@ -10782,9 +10705,6 @@
         <v>275</v>
       </c>
       <c r="DW26" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX26" t="n">
         <v>9614</v>
       </c>
     </row>
@@ -11170,9 +11090,6 @@
         <v>135</v>
       </c>
       <c r="DW27" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX27" t="n">
         <v>7109</v>
       </c>
     </row>
@@ -11558,9 +11475,6 @@
         <v>120</v>
       </c>
       <c r="DW28" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX28" t="n">
         <v>8471</v>
       </c>
     </row>
@@ -11946,9 +11860,6 @@
         <v>255</v>
       </c>
       <c r="DW29" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX29" t="n">
         <v>7500</v>
       </c>
     </row>
@@ -12334,9 +12245,6 @@
         <v>115</v>
       </c>
       <c r="DW30" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX30" t="n">
         <v>9528</v>
       </c>
     </row>
@@ -12722,9 +12630,6 @@
         <v>125</v>
       </c>
       <c r="DW31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX31" t="n">
         <v>10630</v>
       </c>
     </row>
@@ -13110,9 +13015,6 @@
         <v>245</v>
       </c>
       <c r="DW32" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX32" t="n">
         <v>10874</v>
       </c>
     </row>
@@ -13498,9 +13400,6 @@
         <v>150</v>
       </c>
       <c r="DW33" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX33" t="n">
         <v>10666</v>
       </c>
     </row>
@@ -13886,9 +13785,6 @@
         <v>250</v>
       </c>
       <c r="DW34" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX34" t="n">
         <v>12456</v>
       </c>
     </row>
@@ -14274,9 +14170,6 @@
         <v>130</v>
       </c>
       <c r="DW35" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX35" t="n">
         <v>13691</v>
       </c>
     </row>
@@ -14662,9 +14555,6 @@
         <v>360</v>
       </c>
       <c r="DW36" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX36" t="n">
         <v>8648</v>
       </c>
     </row>
@@ -15050,9 +14940,6 @@
         <v>90</v>
       </c>
       <c r="DW37" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX37" t="n">
         <v>6784</v>
       </c>
     </row>
@@ -15438,9 +15325,6 @@
         <v>100</v>
       </c>
       <c r="DW38" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX38" t="n">
         <v>8568</v>
       </c>
     </row>
@@ -15826,9 +15710,6 @@
         <v>340</v>
       </c>
       <c r="DW39" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX39" t="n">
         <v>11377</v>
       </c>
     </row>
@@ -16214,9 +16095,6 @@
         <v>230</v>
       </c>
       <c r="DW40" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX40" t="n">
         <v>13755</v>
       </c>
     </row>
@@ -16602,9 +16480,6 @@
         <v>200</v>
       </c>
       <c r="DW41" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX41" t="n">
         <v>15131</v>
       </c>
     </row>
@@ -16663,7 +16538,7 @@
         <v>0</v>
       </c>
       <c r="R42" t="n">
-        <v>3763</v>
+        <v>3788</v>
       </c>
       <c r="S42" t="n">
         <v>0</v>
@@ -16990,9 +16865,6 @@
         <v>295</v>
       </c>
       <c r="DW42" t="n">
-        <v>25</v>
-      </c>
-      <c r="DX42" t="n">
         <v>14730</v>
       </c>
     </row>
@@ -17378,9 +17250,6 @@
         <v>150</v>
       </c>
       <c r="DW43" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX43" t="n">
         <v>12610</v>
       </c>
     </row>
@@ -17766,9 +17635,6 @@
         <v>120</v>
       </c>
       <c r="DW44" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX44" t="n">
         <v>17534</v>
       </c>
     </row>
@@ -18154,9 +18020,6 @@
         <v>235</v>
       </c>
       <c r="DW45" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX45" t="n">
         <v>13384</v>
       </c>
     </row>
@@ -18542,9 +18405,6 @@
         <v>405</v>
       </c>
       <c r="DW46" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX46" t="n">
         <v>12785</v>
       </c>
     </row>
@@ -18930,9 +18790,6 @@
         <v>290</v>
       </c>
       <c r="DW47" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX47" t="n">
         <v>16316</v>
       </c>
     </row>
@@ -19318,9 +19175,6 @@
         <v>250</v>
       </c>
       <c r="DW48" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX48" t="n">
         <v>12160</v>
       </c>
     </row>
@@ -19706,9 +19560,6 @@
         <v>240</v>
       </c>
       <c r="DW49" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX49" t="n">
         <v>12983</v>
       </c>
     </row>
@@ -20094,9 +19945,6 @@
         <v>215</v>
       </c>
       <c r="DW50" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX50" t="n">
         <v>11689</v>
       </c>
     </row>
@@ -20482,9 +20330,6 @@
         <v>185</v>
       </c>
       <c r="DW51" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX51" t="n">
         <v>14564</v>
       </c>
     </row>
@@ -20870,9 +20715,6 @@
         <v>360</v>
       </c>
       <c r="DW52" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX52" t="n">
         <v>15290</v>
       </c>
     </row>
@@ -21258,9 +21100,6 @@
         <v>390</v>
       </c>
       <c r="DW53" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX53" t="n">
         <v>14760</v>
       </c>
     </row>
@@ -21646,9 +21485,6 @@
         <v>325</v>
       </c>
       <c r="DW54" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX54" t="n">
         <v>17060</v>
       </c>
     </row>
@@ -22034,9 +21870,6 @@
         <v>250</v>
       </c>
       <c r="DW55" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX55" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -22422,9 +22255,6 @@
         <v>575</v>
       </c>
       <c r="DW56" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX56" t="n">
         <v>16605</v>
       </c>
     </row>
@@ -22810,9 +22640,6 @@
         <v>0</v>
       </c>
       <c r="DW57" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX57" t="n">
         <v>12257</v>
       </c>
     </row>
@@ -23198,9 +23025,6 @@
         <v>230</v>
       </c>
       <c r="DW58" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX58" t="n">
         <v>13805</v>
       </c>
     </row>
@@ -23586,9 +23410,6 @@
         <v>225</v>
       </c>
       <c r="DW59" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX59" t="n">
         <v>17125</v>
       </c>
     </row>
@@ -23974,9 +23795,6 @@
         <v>0</v>
       </c>
       <c r="DW60" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX60" t="n">
         <v>14217</v>
       </c>
     </row>
@@ -24362,9 +24180,6 @@
         <v>490</v>
       </c>
       <c r="DW61" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX61" t="n">
         <v>13660</v>
       </c>
     </row>
@@ -24750,9 +24565,6 @@
         <v>160</v>
       </c>
       <c r="DW62" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX62" t="n">
         <v>13706</v>
       </c>
     </row>
@@ -25138,9 +24950,6 @@
         <v>175</v>
       </c>
       <c r="DW63" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX63" t="n">
         <v>12776</v>
       </c>
     </row>
@@ -25199,7 +25008,7 @@
         <v>0</v>
       </c>
       <c r="R64" t="n">
-        <v>2510</v>
+        <v>2525</v>
       </c>
       <c r="S64" t="n">
         <v>0</v>
@@ -25526,9 +25335,6 @@
         <v>270</v>
       </c>
       <c r="DW64" t="n">
-        <v>15</v>
-      </c>
-      <c r="DX64" t="n">
         <v>14345</v>
       </c>
     </row>
@@ -25914,9 +25720,6 @@
         <v>0</v>
       </c>
       <c r="DW65" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX65" t="n">
         <v>15526</v>
       </c>
     </row>
@@ -26302,9 +26105,6 @@
         <v>0</v>
       </c>
       <c r="DW66" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX66" t="n">
         <v>5925</v>
       </c>
     </row>
@@ -26690,9 +26490,6 @@
         <v>0</v>
       </c>
       <c r="DW67" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX67" t="n">
         <v>11805</v>
       </c>
     </row>
@@ -27078,9 +26875,6 @@
         <v>350</v>
       </c>
       <c r="DW68" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX68" t="n">
         <v>12175</v>
       </c>
     </row>
@@ -27466,9 +27260,6 @@
         <v>200</v>
       </c>
       <c r="DW69" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX69" t="n">
         <v>9840</v>
       </c>
     </row>
@@ -27854,9 +27645,6 @@
         <v>470</v>
       </c>
       <c r="DW70" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX70" t="n">
         <v>12013</v>
       </c>
     </row>
@@ -28242,9 +28030,6 @@
         <v>0</v>
       </c>
       <c r="DW71" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX71" t="n">
         <v>12670</v>
       </c>
     </row>
@@ -28630,9 +28415,6 @@
         <v>325</v>
       </c>
       <c r="DW72" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX72" t="n">
         <v>11765</v>
       </c>
     </row>
@@ -29018,9 +28800,6 @@
         <v>145</v>
       </c>
       <c r="DW73" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX73" t="n">
         <v>14015</v>
       </c>
     </row>
@@ -29406,9 +29185,6 @@
         <v>90</v>
       </c>
       <c r="DW74" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX74" t="n">
         <v>11560</v>
       </c>
     </row>
@@ -29794,9 +29570,6 @@
         <v>0</v>
       </c>
       <c r="DW75" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX75" t="n">
         <v>8840</v>
       </c>
     </row>
@@ -30182,9 +29955,6 @@
         <v>0</v>
       </c>
       <c r="DW76" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX76" t="n">
         <v>11850</v>
       </c>
     </row>
@@ -30570,9 +30340,6 @@
         <v>0</v>
       </c>
       <c r="DW77" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX77" t="n">
         <v>9130</v>
       </c>
     </row>
@@ -30958,9 +30725,6 @@
         <v>450</v>
       </c>
       <c r="DW78" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX78" t="n">
         <v>13910</v>
       </c>
     </row>
@@ -31346,9 +31110,6 @@
         <v>0</v>
       </c>
       <c r="DW79" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX79" t="n">
         <v>16004</v>
       </c>
     </row>
@@ -31734,9 +31495,6 @@
         <v>280</v>
       </c>
       <c r="DW80" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX80" t="n">
         <v>15277</v>
       </c>
     </row>
@@ -32122,9 +31880,6 @@
         <v>375</v>
       </c>
       <c r="DW81" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX81" t="n">
         <v>18620</v>
       </c>
     </row>
@@ -32510,9 +32265,6 @@
         <v>0</v>
       </c>
       <c r="DW82" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX82" t="n">
         <v>13578</v>
       </c>
     </row>
@@ -32571,7 +32323,7 @@
         <v>0</v>
       </c>
       <c r="R83" t="n">
-        <v>2505</v>
+        <v>2525</v>
       </c>
       <c r="S83" t="n">
         <v>0</v>
@@ -32898,9 +32650,6 @@
         <v>170</v>
       </c>
       <c r="DW83" t="n">
-        <v>20</v>
-      </c>
-      <c r="DX83" t="n">
         <v>15190</v>
       </c>
     </row>
@@ -33286,9 +33035,6 @@
         <v>0</v>
       </c>
       <c r="DW84" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX84" t="n">
         <v>16001</v>
       </c>
     </row>
@@ -33674,9 +33420,6 @@
         <v>215</v>
       </c>
       <c r="DW85" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX85" t="n">
         <v>17947</v>
       </c>
     </row>
@@ -34062,9 +33805,6 @@
         <v>0</v>
       </c>
       <c r="DW86" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX86" t="n">
         <v>9626</v>
       </c>
     </row>
@@ -34450,9 +34190,6 @@
         <v>95</v>
       </c>
       <c r="DW87" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX87" t="n">
         <v>13102</v>
       </c>
     </row>
@@ -34838,9 +34575,6 @@
         <v>100</v>
       </c>
       <c r="DW88" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX88" t="n">
         <v>22746</v>
       </c>
     </row>
@@ -35226,9 +34960,6 @@
         <v>0</v>
       </c>
       <c r="DW89" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX89" t="n">
         <v>21050</v>
       </c>
     </row>
@@ -35614,9 +35345,6 @@
         <v>140</v>
       </c>
       <c r="DW90" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX90" t="n">
         <v>17690</v>
       </c>
     </row>
@@ -36002,9 +35730,6 @@
         <v>170</v>
       </c>
       <c r="DW91" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX91" t="n">
         <v>18845</v>
       </c>
     </row>
@@ -36390,9 +36115,6 @@
         <v>240</v>
       </c>
       <c r="DW92" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX92" t="n">
         <v>18167</v>
       </c>
     </row>
@@ -36778,9 +36500,6 @@
         <v>265</v>
       </c>
       <c r="DW93" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX93" t="n">
         <v>23259</v>
       </c>
     </row>
@@ -37166,9 +36885,6 @@
         <v>120</v>
       </c>
       <c r="DW94" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX94" t="n">
         <v>23761</v>
       </c>
     </row>
@@ -37554,9 +37270,6 @@
         <v>440</v>
       </c>
       <c r="DW95" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX95" t="n">
         <v>20768</v>
       </c>
     </row>
@@ -37615,7 +37328,7 @@
         <v>0</v>
       </c>
       <c r="R96" t="n">
-        <v>3658</v>
+        <v>3678</v>
       </c>
       <c r="S96" t="n">
         <v>0</v>
@@ -37942,9 +37655,6 @@
         <v>185</v>
       </c>
       <c r="DW96" t="n">
-        <v>20</v>
-      </c>
-      <c r="DX96" t="n">
         <v>20799</v>
       </c>
     </row>
@@ -38330,9 +38040,6 @@
         <v>0</v>
       </c>
       <c r="DW97" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX97" t="n">
         <v>16576</v>
       </c>
     </row>
@@ -38718,9 +38425,6 @@
         <v>200</v>
       </c>
       <c r="DW98" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX98" t="n">
         <v>16360</v>
       </c>
     </row>
@@ -39106,9 +38810,6 @@
         <v>40</v>
       </c>
       <c r="DW99" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX99" t="n">
         <v>21630</v>
       </c>
     </row>
@@ -39494,9 +39195,6 @@
         <v>90</v>
       </c>
       <c r="DW100" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX100" t="n">
         <v>20500</v>
       </c>
     </row>
@@ -39882,9 +39580,6 @@
         <v>325</v>
       </c>
       <c r="DW101" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX101" t="n">
         <v>19064</v>
       </c>
     </row>
@@ -40270,9 +39965,6 @@
         <v>0</v>
       </c>
       <c r="DW102" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX102" t="n">
         <v>21982</v>
       </c>
     </row>
@@ -40658,9 +40350,6 @@
         <v>187</v>
       </c>
       <c r="DW103" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX103" t="n">
         <v>24960</v>
       </c>
     </row>
@@ -41046,9 +40735,6 @@
         <v>150</v>
       </c>
       <c r="DW104" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX104" t="n">
         <v>18055</v>
       </c>
     </row>
@@ -41434,9 +41120,6 @@
         <v>445</v>
       </c>
       <c r="DW105" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX105" t="n">
         <v>24501</v>
       </c>
     </row>
@@ -41822,9 +41505,6 @@
         <v>0</v>
       </c>
       <c r="DW106" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX106" t="n">
         <v>17565</v>
       </c>
     </row>
@@ -42210,9 +41890,6 @@
         <v>620</v>
       </c>
       <c r="DW107" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX107" t="n">
         <v>23263</v>
       </c>
     </row>
@@ -42598,9 +42275,6 @@
         <v>280</v>
       </c>
       <c r="DW108" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX108" t="n">
         <v>18300</v>
       </c>
     </row>
@@ -42986,9 +42660,6 @@
         <v>260</v>
       </c>
       <c r="DW109" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX109" t="n">
         <v>18226</v>
       </c>
     </row>
@@ -43374,9 +43045,6 @@
         <v>255</v>
       </c>
       <c r="DW110" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX110" t="n">
         <v>19982</v>
       </c>
     </row>
@@ -43762,9 +43430,6 @@
         <v>390</v>
       </c>
       <c r="DW111" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX111" t="n">
         <v>21041</v>
       </c>
     </row>
@@ -44150,9 +43815,6 @@
         <v>200</v>
       </c>
       <c r="DW112" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX112" t="n">
         <v>20551</v>
       </c>
     </row>
@@ -44538,9 +44200,6 @@
         <v>390</v>
       </c>
       <c r="DW113" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX113" t="n">
         <v>25985</v>
       </c>
     </row>
@@ -44926,9 +44585,6 @@
         <v>210</v>
       </c>
       <c r="DW114" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX114" t="n">
         <v>20431</v>
       </c>
     </row>
@@ -45314,9 +44970,6 @@
         <v>390</v>
       </c>
       <c r="DW115" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX115" t="n">
         <v>22304</v>
       </c>
     </row>
@@ -45702,9 +45355,6 @@
         <v>160</v>
       </c>
       <c r="DW116" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX116" t="n">
         <v>24250</v>
       </c>
     </row>
@@ -46090,9 +45740,6 @@
         <v>520</v>
       </c>
       <c r="DW117" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX117" t="n">
         <v>21683</v>
       </c>
     </row>
@@ -46478,9 +46125,6 @@
         <v>70</v>
       </c>
       <c r="DW118" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX118" t="n">
         <v>23851</v>
       </c>
     </row>
@@ -46539,7 +46183,7 @@
         <v>0</v>
       </c>
       <c r="R119" t="n">
-        <v>5018</v>
+        <v>5028</v>
       </c>
       <c r="S119" t="n">
         <v>0</v>
@@ -46866,9 +46510,6 @@
         <v>510</v>
       </c>
       <c r="DW119" t="n">
-        <v>10</v>
-      </c>
-      <c r="DX119" t="n">
         <v>22607</v>
       </c>
     </row>
@@ -47254,9 +46895,6 @@
         <v>470</v>
       </c>
       <c r="DW120" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX120" t="n">
         <v>20266</v>
       </c>
     </row>
@@ -47642,9 +47280,6 @@
         <v>135</v>
       </c>
       <c r="DW121" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX121" t="n">
         <v>20384</v>
       </c>
     </row>
@@ -48030,9 +47665,6 @@
         <v>95</v>
       </c>
       <c r="DW122" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX122" t="n">
         <v>19150</v>
       </c>
     </row>
@@ -48418,9 +48050,6 @@
         <v>165</v>
       </c>
       <c r="DW123" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX123" t="n">
         <v>18144</v>
       </c>
     </row>
@@ -48806,9 +48435,6 @@
         <v>350</v>
       </c>
       <c r="DW124" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX124" t="n">
         <v>26985</v>
       </c>
     </row>
@@ -49194,9 +48820,6 @@
         <v>60</v>
       </c>
       <c r="DW125" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX125" t="n">
         <v>27151</v>
       </c>
     </row>
@@ -49582,9 +49205,6 @@
         <v>115</v>
       </c>
       <c r="DW126" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX126" t="n">
         <v>20765</v>
       </c>
     </row>
@@ -49970,9 +49590,6 @@
         <v>282</v>
       </c>
       <c r="DW127" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX127" t="n">
         <v>23443</v>
       </c>
     </row>
@@ -50358,9 +49975,6 @@
         <v>485</v>
       </c>
       <c r="DW128" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX128" t="n">
         <v>22680</v>
       </c>
     </row>
@@ -50746,9 +50360,6 @@
         <v>350</v>
       </c>
       <c r="DW129" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX129" t="n">
         <v>25127</v>
       </c>
     </row>
@@ -51134,9 +50745,6 @@
         <v>130</v>
       </c>
       <c r="DW130" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX130" t="n">
         <v>25506</v>
       </c>
     </row>
@@ -51522,9 +51130,6 @@
         <v>372</v>
       </c>
       <c r="DW131" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX131" t="n">
         <v>21978</v>
       </c>
     </row>
@@ -51910,9 +51515,6 @@
         <v>445</v>
       </c>
       <c r="DW132" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX132" t="n">
         <v>20167</v>
       </c>
     </row>
@@ -52298,9 +51900,6 @@
         <v>185</v>
       </c>
       <c r="DW133" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX133" t="n">
         <v>18881</v>
       </c>
     </row>
@@ -52686,9 +52285,6 @@
         <v>240</v>
       </c>
       <c r="DW134" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX134" t="n">
         <v>22058</v>
       </c>
     </row>
@@ -53074,9 +52670,6 @@
         <v>185</v>
       </c>
       <c r="DW135" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX135" t="n">
         <v>20695</v>
       </c>
     </row>
@@ -53462,9 +53055,6 @@
         <v>335</v>
       </c>
       <c r="DW136" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX136" t="n">
         <v>25977</v>
       </c>
     </row>
@@ -53850,9 +53440,6 @@
         <v>250</v>
       </c>
       <c r="DW137" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX137" t="n">
         <v>27829</v>
       </c>
     </row>
@@ -53911,7 +53498,7 @@
         <v>0</v>
       </c>
       <c r="R138" t="n">
-        <v>3655</v>
+        <v>3657</v>
       </c>
       <c r="S138" t="n">
         <v>65</v>
@@ -54103,7 +53690,7 @@
         <v>0</v>
       </c>
       <c r="CD138" t="n">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="CE138" t="n">
         <v>138</v>
@@ -54238,9 +53825,6 @@
         <v>150</v>
       </c>
       <c r="DW138" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX138" t="n">
         <v>20343</v>
       </c>
     </row>
@@ -54260,7 +53844,7 @@
         <v>0</v>
       </c>
       <c r="E139" t="n">
-        <v>130</v>
+        <v>250</v>
       </c>
       <c r="F139" t="n">
         <v>0</v>
@@ -54299,7 +53883,7 @@
         <v>35</v>
       </c>
       <c r="R139" t="n">
-        <v>4164</v>
+        <v>4514</v>
       </c>
       <c r="S139" t="n">
         <v>0</v>
@@ -54317,7 +53901,7 @@
         <v>120</v>
       </c>
       <c r="X139" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="Y139" t="n">
         <v>0</v>
@@ -54329,7 +53913,7 @@
         <v>0</v>
       </c>
       <c r="AB139" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="AC139" t="n">
         <v>0</v>
@@ -54362,7 +53946,7 @@
         <v>0</v>
       </c>
       <c r="AM139" t="n">
-        <v>170</v>
+        <v>235</v>
       </c>
       <c r="AN139" t="n">
         <v>90</v>
@@ -54434,7 +54018,7 @@
         <v>50</v>
       </c>
       <c r="BK139" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="BL139" t="n">
         <v>260</v>
@@ -54452,7 +54036,7 @@
         <v>0</v>
       </c>
       <c r="BQ139" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="BR139" t="n">
         <v>215</v>
@@ -54491,10 +54075,10 @@
         <v>0</v>
       </c>
       <c r="CD139" t="n">
-        <v>280</v>
+        <v>380</v>
       </c>
       <c r="CE139" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
       <c r="CF139" t="n">
         <v>0</v>
@@ -54533,13 +54117,13 @@
         <v>0</v>
       </c>
       <c r="CR139" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="CS139" t="n">
         <v>0</v>
       </c>
       <c r="CT139" t="n">
-        <v>310</v>
+        <v>640</v>
       </c>
       <c r="CU139" t="n">
         <v>75</v>
@@ -54551,25 +54135,25 @@
         <v>0</v>
       </c>
       <c r="CX139" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="CY139" t="n">
         <v>64</v>
       </c>
       <c r="CZ139" t="n">
-        <v>165</v>
+        <v>495</v>
       </c>
       <c r="DA139" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="DB139" t="n">
-        <v>795</v>
+        <v>1610</v>
       </c>
       <c r="DC139" t="n">
         <v>0</v>
       </c>
       <c r="DD139" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="DE139" t="n">
         <v>0</v>
@@ -54587,7 +54171,7 @@
         <v>205</v>
       </c>
       <c r="DJ139" t="n">
-        <v>0</v>
+        <v>745</v>
       </c>
       <c r="DK139" t="n">
         <v>200</v>
@@ -54611,7 +54195,7 @@
         <v>0</v>
       </c>
       <c r="DR139" t="n">
-        <v>700</v>
+        <v>923</v>
       </c>
       <c r="DS139" t="n">
         <v>0</v>
@@ -54626,10 +54210,7 @@
         <v>310</v>
       </c>
       <c r="DW139" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX139" t="n">
-        <v>22927</v>
+        <v>26657</v>
       </c>
     </row>
     <row r="140">
@@ -54648,7 +54229,7 @@
         <v>150</v>
       </c>
       <c r="E140" t="n">
-        <v>71345</v>
+        <v>71465</v>
       </c>
       <c r="F140" t="n">
         <v>500</v>
@@ -54687,7 +54268,7 @@
         <v>107</v>
       </c>
       <c r="R140" t="n">
-        <v>428686</v>
+        <v>429168</v>
       </c>
       <c r="S140" t="n">
         <v>925</v>
@@ -54705,7 +54286,7 @@
         <v>23953</v>
       </c>
       <c r="X140" t="n">
-        <v>4542</v>
+        <v>4712</v>
       </c>
       <c r="Y140" t="n">
         <v>2947</v>
@@ -54717,7 +54298,7 @@
         <v>2</v>
       </c>
       <c r="AB140" t="n">
-        <v>8979</v>
+        <v>9129</v>
       </c>
       <c r="AC140" t="n">
         <v>212</v>
@@ -54750,7 +54331,7 @@
         <v>374</v>
       </c>
       <c r="AM140" t="n">
-        <v>50594</v>
+        <v>50659</v>
       </c>
       <c r="AN140" t="n">
         <v>4755</v>
@@ -54822,7 +54403,7 @@
         <v>1007</v>
       </c>
       <c r="BK140" t="n">
-        <v>650</v>
+        <v>660</v>
       </c>
       <c r="BL140" t="n">
         <v>47345</v>
@@ -54840,7 +54421,7 @@
         <v>7365</v>
       </c>
       <c r="BQ140" t="n">
-        <v>94080</v>
+        <v>94095</v>
       </c>
       <c r="BR140" t="n">
         <v>22072</v>
@@ -54879,10 +54460,10 @@
         <v>435</v>
       </c>
       <c r="CD140" t="n">
-        <v>15275</v>
+        <v>15373</v>
       </c>
       <c r="CE140" t="n">
-        <v>5629</v>
+        <v>5771</v>
       </c>
       <c r="CF140" t="n">
         <v>145</v>
@@ -54921,13 +54502,13 @@
         <v>277</v>
       </c>
       <c r="CR140" t="n">
-        <v>11874</v>
+        <v>11904</v>
       </c>
       <c r="CS140" t="n">
         <v>2</v>
       </c>
       <c r="CT140" t="n">
-        <v>64775</v>
+        <v>65105</v>
       </c>
       <c r="CU140" t="n">
         <v>2384</v>
@@ -54939,25 +54520,25 @@
         <v>2698</v>
       </c>
       <c r="CX140" t="n">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="CY140" t="n">
         <v>8936</v>
       </c>
       <c r="CZ140" t="n">
-        <v>18166</v>
+        <v>18496</v>
       </c>
       <c r="DA140" t="n">
-        <v>13716</v>
+        <v>13766</v>
       </c>
       <c r="DB140" t="n">
-        <v>217038</v>
+        <v>217853</v>
       </c>
       <c r="DC140" t="n">
         <v>1030</v>
       </c>
       <c r="DD140" t="n">
-        <v>1281</v>
+        <v>1351</v>
       </c>
       <c r="DE140" t="n">
         <v>1485</v>
@@ -54975,7 +54556,7 @@
         <v>23863</v>
       </c>
       <c r="DJ140" t="n">
-        <v>99229</v>
+        <v>99974</v>
       </c>
       <c r="DK140" t="n">
         <v>1240</v>
@@ -54999,7 +54580,7 @@
         <v>7725</v>
       </c>
       <c r="DR140" t="n">
-        <v>57518</v>
+        <v>57741</v>
       </c>
       <c r="DS140" t="n">
         <v>1450</v>
@@ -55014,10 +54595,7 @@
         <v>27338</v>
       </c>
       <c r="DW140" t="n">
-        <v>130</v>
-      </c>
-      <c r="DX140" t="n">
-        <v>2058792</v>
+        <v>2062522</v>
       </c>
     </row>
   </sheetData>
@@ -55350,10 +54928,10 @@
         <v>1497</v>
       </c>
       <c r="N6" t="n">
-        <v>3363</v>
+        <v>3388</v>
       </c>
       <c r="O6" t="n">
-        <v>9190</v>
+        <v>9215</v>
       </c>
     </row>
     <row r="7">
@@ -55742,10 +55320,10 @@
         <v>21112</v>
       </c>
       <c r="N14" t="n">
-        <v>41697</v>
+        <v>41722</v>
       </c>
       <c r="O14" t="n">
-        <v>117677</v>
+        <v>117702</v>
       </c>
     </row>
   </sheetData>
@@ -56708,10 +56286,10 @@
         <v>1165</v>
       </c>
       <c r="N4" t="n">
-        <v>2510</v>
+        <v>2525</v>
       </c>
       <c r="O4" t="n">
-        <v>9695</v>
+        <v>9710</v>
       </c>
     </row>
     <row r="5">
@@ -57198,10 +56776,10 @@
         <v>15805</v>
       </c>
       <c r="N14" t="n">
-        <v>23257</v>
+        <v>23272</v>
       </c>
       <c r="O14" t="n">
-        <v>90008</v>
+        <v>90023</v>
       </c>
     </row>
   </sheetData>
@@ -57779,10 +57357,10 @@
         <v>2095</v>
       </c>
       <c r="N11" t="n">
-        <v>2355</v>
+        <v>2375</v>
       </c>
       <c r="O11" t="n">
-        <v>10435</v>
+        <v>10455</v>
       </c>
     </row>
     <row r="12">
@@ -57926,10 +57504,10 @@
         <v>18542</v>
       </c>
       <c r="N14" t="n">
-        <v>26144</v>
+        <v>26164</v>
       </c>
       <c r="O14" t="n">
-        <v>102866</v>
+        <v>102886</v>
       </c>
     </row>
   </sheetData>
@@ -58556,10 +58134,10 @@
         <v>2384</v>
       </c>
       <c r="N12" t="n">
-        <v>3088</v>
+        <v>3108</v>
       </c>
       <c r="O12" t="n">
-        <v>12143</v>
+        <v>12163</v>
       </c>
     </row>
     <row r="13">
@@ -58654,10 +58232,10 @@
         <v>22238</v>
       </c>
       <c r="N14" t="n">
-        <v>34219</v>
+        <v>34239</v>
       </c>
       <c r="O14" t="n">
-        <v>125343</v>
+        <v>125363</v>
       </c>
     </row>
   </sheetData>
@@ -59963,10 +59541,10 @@
         <v>1554</v>
       </c>
       <c r="N11" t="n">
-        <v>4468</v>
+        <v>4478</v>
       </c>
       <c r="O11" t="n">
-        <v>12972</v>
+        <v>12982</v>
       </c>
     </row>
     <row r="12">
@@ -60110,10 +59688,10 @@
         <v>27438</v>
       </c>
       <c r="N14" t="n">
-        <v>39604</v>
+        <v>39614</v>
       </c>
       <c r="O14" t="n">
-        <v>158260</v>
+        <v>158270</v>
       </c>
     </row>
   </sheetData>
@@ -61174,10 +60752,10 @@
         <v>2564</v>
       </c>
       <c r="N6" t="n">
-        <v>3220</v>
+        <v>3222</v>
       </c>
       <c r="O6" t="n">
-        <v>12471</v>
+        <v>12473</v>
       </c>
     </row>
     <row r="7">
@@ -61187,10 +60765,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>795</v>
+        <v>1610</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>745</v>
       </c>
       <c r="D7" t="n">
         <v>425</v>
@@ -61220,13 +60798,13 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>780</v>
+        <v>915</v>
       </c>
       <c r="N7" t="n">
-        <v>4164</v>
+        <v>4514</v>
       </c>
       <c r="O7" t="n">
-        <v>8349</v>
+        <v>10394</v>
       </c>
     </row>
     <row r="8">
@@ -61236,10 +60814,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12965</v>
+        <v>13780</v>
       </c>
       <c r="C8" t="n">
-        <v>4720</v>
+        <v>5465</v>
       </c>
       <c r="D8" t="n">
         <v>5000</v>
@@ -61269,13 +60847,13 @@
         <v>2690</v>
       </c>
       <c r="M8" t="n">
-        <v>12326</v>
+        <v>12461</v>
       </c>
       <c r="N8" t="n">
-        <v>20805</v>
+        <v>21157</v>
       </c>
       <c r="O8" t="n">
-        <v>81134</v>
+        <v>83181</v>
       </c>
     </row>
   </sheetData>
@@ -62681,7 +62259,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>795</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="140">
@@ -62691,7 +62269,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>217038</v>
+        <v>217853</v>
       </c>
     </row>
     <row r="142">
@@ -62799,7 +62377,7 @@
         <v>2026</v>
       </c>
       <c r="B154" t="n">
-        <v>12965</v>
+        <v>13780</v>
       </c>
     </row>
     <row r="155">
@@ -62809,7 +62387,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>217038</v>
+        <v>217853</v>
       </c>
     </row>
   </sheetData>
@@ -63244,7 +62822,7 @@
         <v>45</v>
       </c>
       <c r="E7" t="n">
-        <v>1946</v>
+        <v>1971</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -63277,7 +62855,7 @@
         <v>30</v>
       </c>
       <c r="P7" t="n">
-        <v>1257</v>
+        <v>1232</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -63610,7 +63188,7 @@
         <v>45</v>
       </c>
       <c r="E13" t="n">
-        <v>2615</v>
+        <v>2630</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -63643,7 +63221,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>926</v>
+        <v>911</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
@@ -65379,7 +64957,7 @@
         <v>485</v>
       </c>
       <c r="E42" t="n">
-        <v>7768</v>
+        <v>7793</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -65412,7 +64990,7 @@
         <v>275</v>
       </c>
       <c r="P42" t="n">
-        <v>2517</v>
+        <v>2492</v>
       </c>
       <c r="Q42" t="n">
         <v>0</v>
@@ -66721,7 +66299,7 @@
         <v>990</v>
       </c>
       <c r="E64" t="n">
-        <v>4360</v>
+        <v>4375</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
@@ -66754,7 +66332,7 @@
         <v>165</v>
       </c>
       <c r="P64" t="n">
-        <v>3350</v>
+        <v>3335</v>
       </c>
       <c r="Q64" t="n">
         <v>925</v>
@@ -67880,7 +67458,7 @@
         <v>110</v>
       </c>
       <c r="E83" t="n">
-        <v>5573</v>
+        <v>5593</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -67898,13 +67476,13 @@
         <v>0</v>
       </c>
       <c r="K83" t="n">
-        <v>1070</v>
+        <v>990</v>
       </c>
       <c r="L83" t="n">
         <v>205</v>
       </c>
       <c r="M83" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="N83" t="n">
         <v>0</v>
@@ -67913,7 +67491,7 @@
         <v>0</v>
       </c>
       <c r="P83" t="n">
-        <v>3777</v>
+        <v>3757</v>
       </c>
       <c r="Q83" t="n">
         <v>0</v>
@@ -67959,13 +67537,13 @@
         <v>0</v>
       </c>
       <c r="K84" t="n">
-        <v>200</v>
+        <v>125</v>
       </c>
       <c r="L84" t="n">
         <v>155</v>
       </c>
       <c r="M84" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="N84" t="n">
         <v>0</v>
@@ -68020,13 +67598,13 @@
         <v>0</v>
       </c>
       <c r="K85" t="n">
-        <v>991</v>
+        <v>891</v>
       </c>
       <c r="L85" t="n">
         <v>210</v>
       </c>
       <c r="M85" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="N85" t="n">
         <v>25</v>
@@ -68142,13 +67720,13 @@
         <v>0</v>
       </c>
       <c r="K87" t="n">
-        <v>1425</v>
+        <v>1395</v>
       </c>
       <c r="L87" t="n">
         <v>260</v>
       </c>
       <c r="M87" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="N87" t="n">
         <v>0</v>
@@ -68203,13 +67781,13 @@
         <v>0</v>
       </c>
       <c r="K88" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L88" t="n">
         <v>405</v>
       </c>
       <c r="M88" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="N88" t="n">
         <v>0</v>
@@ -68264,13 +67842,13 @@
         <v>0</v>
       </c>
       <c r="K89" t="n">
-        <v>2100</v>
+        <v>1920</v>
       </c>
       <c r="L89" t="n">
         <v>210</v>
       </c>
       <c r="M89" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="N89" t="n">
         <v>0</v>
@@ -68325,13 +67903,13 @@
         <v>0</v>
       </c>
       <c r="K90" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="L90" t="n">
         <v>205</v>
       </c>
       <c r="M90" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="N90" t="n">
         <v>0</v>
@@ -68447,13 +68025,13 @@
         <v>0</v>
       </c>
       <c r="K92" t="n">
-        <v>493</v>
+        <v>453</v>
       </c>
       <c r="L92" t="n">
         <v>415</v>
       </c>
       <c r="M92" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="N92" t="n">
         <v>0</v>
@@ -68508,13 +68086,13 @@
         <v>0</v>
       </c>
       <c r="K93" t="n">
-        <v>1360</v>
+        <v>1290</v>
       </c>
       <c r="L93" t="n">
         <v>0</v>
       </c>
       <c r="M93" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="N93" t="n">
         <v>0</v>
@@ -68630,13 +68208,13 @@
         <v>0</v>
       </c>
       <c r="K95" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="L95" t="n">
         <v>367</v>
       </c>
       <c r="M95" t="n">
-        <v>126</v>
+        <v>166</v>
       </c>
       <c r="N95" t="n">
         <v>0</v>
@@ -68673,7 +68251,7 @@
         <v>515</v>
       </c>
       <c r="E96" t="n">
-        <v>7375</v>
+        <v>7395</v>
       </c>
       <c r="F96" t="n">
         <v>0</v>
@@ -68706,7 +68284,7 @@
         <v>352</v>
       </c>
       <c r="P96" t="n">
-        <v>4034</v>
+        <v>4014</v>
       </c>
       <c r="Q96" t="n">
         <v>210</v>
@@ -68813,13 +68391,13 @@
         <v>85</v>
       </c>
       <c r="K98" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="L98" t="n">
         <v>354</v>
       </c>
       <c r="M98" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="N98" t="n">
         <v>0</v>
@@ -68935,13 +68513,13 @@
         <v>0</v>
       </c>
       <c r="K100" t="n">
-        <v>975</v>
+        <v>925</v>
       </c>
       <c r="L100" t="n">
         <v>284</v>
       </c>
       <c r="M100" t="n">
-        <v>127</v>
+        <v>177</v>
       </c>
       <c r="N100" t="n">
         <v>0</v>
@@ -69057,13 +68635,13 @@
         <v>75</v>
       </c>
       <c r="K102" t="n">
-        <v>745</v>
+        <v>675</v>
       </c>
       <c r="L102" t="n">
         <v>313</v>
       </c>
       <c r="M102" t="n">
-        <v>128</v>
+        <v>198</v>
       </c>
       <c r="N102" t="n">
         <v>0</v>
@@ -69118,13 +68696,13 @@
         <v>0</v>
       </c>
       <c r="K103" t="n">
-        <v>1847</v>
+        <v>1780</v>
       </c>
       <c r="L103" t="n">
         <v>440</v>
       </c>
       <c r="M103" t="n">
-        <v>138</v>
+        <v>205</v>
       </c>
       <c r="N103" t="n">
         <v>0</v>
@@ -69301,13 +68879,13 @@
         <v>163</v>
       </c>
       <c r="K106" t="n">
-        <v>862</v>
+        <v>762</v>
       </c>
       <c r="L106" t="n">
         <v>378</v>
       </c>
       <c r="M106" t="n">
-        <v>128</v>
+        <v>228</v>
       </c>
       <c r="N106" t="n">
         <v>0</v>
@@ -69423,13 +69001,13 @@
         <v>0</v>
       </c>
       <c r="K108" t="n">
-        <v>1015</v>
+        <v>955</v>
       </c>
       <c r="L108" t="n">
         <v>439</v>
       </c>
       <c r="M108" t="n">
-        <v>137</v>
+        <v>197</v>
       </c>
       <c r="N108" t="n">
         <v>0</v>
@@ -69606,13 +69184,13 @@
         <v>45</v>
       </c>
       <c r="K111" t="n">
-        <v>2026</v>
+        <v>1936</v>
       </c>
       <c r="L111" t="n">
         <v>414</v>
       </c>
       <c r="M111" t="n">
-        <v>104</v>
+        <v>194</v>
       </c>
       <c r="N111" t="n">
         <v>0</v>
@@ -69850,13 +69428,13 @@
         <v>90</v>
       </c>
       <c r="K115" t="n">
-        <v>1005</v>
+        <v>940</v>
       </c>
       <c r="L115" t="n">
         <v>629</v>
       </c>
       <c r="M115" t="n">
-        <v>148</v>
+        <v>213</v>
       </c>
       <c r="N115" t="n">
         <v>0</v>
@@ -69972,13 +69550,13 @@
         <v>302</v>
       </c>
       <c r="K117" t="n">
-        <v>1050</v>
+        <v>910</v>
       </c>
       <c r="L117" t="n">
         <v>464</v>
       </c>
       <c r="M117" t="n">
-        <v>131</v>
+        <v>271</v>
       </c>
       <c r="N117" t="n">
         <v>0</v>
@@ -70076,7 +69654,7 @@
         <v>830</v>
       </c>
       <c r="E119" t="n">
-        <v>11966</v>
+        <v>11976</v>
       </c>
       <c r="F119" t="n">
         <v>197</v>
@@ -70094,13 +69672,13 @@
         <v>100</v>
       </c>
       <c r="K119" t="n">
-        <v>1449</v>
+        <v>1364</v>
       </c>
       <c r="L119" t="n">
         <v>506</v>
       </c>
       <c r="M119" t="n">
-        <v>145</v>
+        <v>230</v>
       </c>
       <c r="N119" t="n">
         <v>0</v>
@@ -70109,7 +69687,7 @@
         <v>165</v>
       </c>
       <c r="P119" t="n">
-        <v>3254</v>
+        <v>3244</v>
       </c>
       <c r="Q119" t="n">
         <v>270</v>
@@ -70216,13 +69794,13 @@
         <v>255</v>
       </c>
       <c r="K121" t="n">
-        <v>1608</v>
+        <v>1518</v>
       </c>
       <c r="L121" t="n">
         <v>394</v>
       </c>
       <c r="M121" t="n">
-        <v>146</v>
+        <v>236</v>
       </c>
       <c r="N121" t="n">
         <v>0</v>
@@ -70399,13 +69977,13 @@
         <v>144</v>
       </c>
       <c r="K124" t="n">
-        <v>2475</v>
+        <v>2385</v>
       </c>
       <c r="L124" t="n">
         <v>308</v>
       </c>
       <c r="M124" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="N124" t="n">
         <v>0</v>
@@ -70521,13 +70099,13 @@
         <v>0</v>
       </c>
       <c r="K126" t="n">
-        <v>1120</v>
+        <v>1000</v>
       </c>
       <c r="L126" t="n">
         <v>0</v>
       </c>
       <c r="M126" t="n">
-        <v>148</v>
+        <v>268</v>
       </c>
       <c r="N126" t="n">
         <v>0</v>
@@ -70643,13 +70221,13 @@
         <v>135</v>
       </c>
       <c r="K128" t="n">
-        <v>1005</v>
+        <v>870</v>
       </c>
       <c r="L128" t="n">
         <v>282</v>
       </c>
       <c r="M128" t="n">
-        <v>129</v>
+        <v>264</v>
       </c>
       <c r="N128" t="n">
         <v>0</v>
@@ -70826,13 +70404,13 @@
         <v>411</v>
       </c>
       <c r="K131" t="n">
-        <v>1779</v>
+        <v>1624</v>
       </c>
       <c r="L131" t="n">
         <v>240</v>
       </c>
       <c r="M131" t="n">
-        <v>149</v>
+        <v>304</v>
       </c>
       <c r="N131" t="n">
         <v>0</v>
@@ -70948,13 +70526,13 @@
         <v>0</v>
       </c>
       <c r="K133" t="n">
-        <v>1923</v>
+        <v>1803</v>
       </c>
       <c r="L133" t="n">
         <v>277</v>
       </c>
       <c r="M133" t="n">
-        <v>108</v>
+        <v>228</v>
       </c>
       <c r="N133" t="n">
         <v>0</v>
@@ -71070,13 +70648,13 @@
         <v>0</v>
       </c>
       <c r="K135" t="n">
-        <v>1795</v>
+        <v>1710</v>
       </c>
       <c r="L135" t="n">
         <v>250</v>
       </c>
       <c r="M135" t="n">
-        <v>133</v>
+        <v>218</v>
       </c>
       <c r="N135" t="n">
         <v>0</v>
@@ -71192,13 +70770,13 @@
         <v>314</v>
       </c>
       <c r="K137" t="n">
-        <v>3060</v>
+        <v>2965</v>
       </c>
       <c r="L137" t="n">
         <v>708</v>
       </c>
       <c r="M137" t="n">
-        <v>159</v>
+        <v>254</v>
       </c>
       <c r="N137" t="n">
         <v>0</v>
@@ -71235,7 +70813,7 @@
         <v>935</v>
       </c>
       <c r="E138" t="n">
-        <v>6856</v>
+        <v>6858</v>
       </c>
       <c r="F138" t="n">
         <v>0</v>
@@ -71268,7 +70846,7 @@
         <v>70</v>
       </c>
       <c r="P138" t="n">
-        <v>4756</v>
+        <v>4754</v>
       </c>
       <c r="Q138" t="n">
         <v>127</v>
@@ -71293,22 +70871,22 @@
         <v>255</v>
       </c>
       <c r="D139" t="n">
-        <v>290</v>
+        <v>670</v>
       </c>
       <c r="E139" t="n">
-        <v>16175</v>
+        <v>17173</v>
       </c>
       <c r="F139" t="n">
         <v>0</v>
       </c>
       <c r="G139" t="n">
-        <v>339</v>
+        <v>754</v>
       </c>
       <c r="H139" t="n">
         <v>75</v>
       </c>
       <c r="I139" t="n">
-        <v>1090</v>
+        <v>1905</v>
       </c>
       <c r="J139" t="n">
         <v>0</v>
@@ -71320,7 +70898,7 @@
         <v>269</v>
       </c>
       <c r="M139" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
       <c r="N139" t="n">
         <v>0</v>
@@ -71329,7 +70907,7 @@
         <v>0</v>
       </c>
       <c r="P139" t="n">
-        <v>1600</v>
+        <v>2580</v>
       </c>
       <c r="Q139" t="n">
         <v>0</v>
@@ -71338,7 +70916,7 @@
         <v>1410</v>
       </c>
       <c r="S139" t="n">
-        <v>22927</v>
+        <v>26657</v>
       </c>
     </row>
     <row r="140">
@@ -71354,34 +70932,34 @@
         <v>17331</v>
       </c>
       <c r="D140" t="n">
-        <v>61678</v>
+        <v>62058</v>
       </c>
       <c r="E140" t="n">
-        <v>850112</v>
+        <v>851242</v>
       </c>
       <c r="F140" t="n">
         <v>5932</v>
       </c>
       <c r="G140" t="n">
-        <v>33600</v>
+        <v>34015</v>
       </c>
       <c r="H140" t="n">
         <v>7499</v>
       </c>
       <c r="I140" t="n">
-        <v>282329</v>
+        <v>283144</v>
       </c>
       <c r="J140" t="n">
         <v>4939</v>
       </c>
       <c r="K140" t="n">
-        <v>111442</v>
+        <v>109060</v>
       </c>
       <c r="L140" t="n">
         <v>35385</v>
       </c>
       <c r="M140" t="n">
-        <v>5629</v>
+        <v>8153</v>
       </c>
       <c r="N140" t="n">
         <v>42</v>
@@ -71390,7 +70968,7 @@
         <v>22052</v>
       </c>
       <c r="P140" t="n">
-        <v>419016</v>
+        <v>419864</v>
       </c>
       <c r="Q140" t="n">
         <v>36635</v>
@@ -71399,7 +70977,7 @@
         <v>87453</v>
       </c>
       <c r="S140" t="n">
-        <v>2058792</v>
+        <v>2062522</v>
       </c>
     </row>
   </sheetData>
@@ -71413,7 +70991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B154"/>
+  <dimension ref="A1:B155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72801,129 +72379,139 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B139" t="n">
-        <v>99229</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
+      <c r="B140" t="n">
+        <v>99974</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
+      <c r="B142" t="inlineStr">
         <is>
           <t>Gallons</t>
         </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B142" t="n">
-        <v>4620</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B143" t="n">
-        <v>9287</v>
+        <v>4620</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="B144" t="n">
-        <v>9052</v>
+        <v>9287</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="B145" t="n">
-        <v>11885</v>
+        <v>9052</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="B146" t="n">
-        <v>10945</v>
+        <v>11885</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B147" t="n">
-        <v>5985</v>
+        <v>10945</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B148" t="n">
-        <v>7702</v>
+        <v>5985</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B149" t="n">
-        <v>7774</v>
+        <v>7702</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B150" t="n">
-        <v>7025</v>
+        <v>7774</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B151" t="n">
-        <v>9804</v>
+        <v>7025</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B152" t="n">
-        <v>10430</v>
+        <v>9804</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B153" t="n">
+        <v>10430</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
         <v>2026</v>
       </c>
-      <c r="B153" t="n">
-        <v>4720</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
+      <c r="B154" t="n">
+        <v>5465</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B154" t="n">
-        <v>99229</v>
+      <c r="B155" t="n">
+        <v>99974</v>
       </c>
     </row>
   </sheetData>
@@ -82985,7 +82573,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1581</v>
+        <v>1606</v>
       </c>
       <c r="C7" t="n">
         <v>830</v>
@@ -83006,7 +82594,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>765</v>
+        <v>740</v>
       </c>
       <c r="J7" t="n">
         <v>470</v>
@@ -83297,7 +82885,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2077</v>
+        <v>2092</v>
       </c>
       <c r="C13" t="n">
         <v>482</v>
@@ -83318,7 +82906,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>788</v>
+        <v>773</v>
       </c>
       <c r="J13" t="n">
         <v>865</v>
@@ -84805,7 +84393,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3363</v>
+        <v>3388</v>
       </c>
       <c r="C42" t="n">
         <v>1497</v>
@@ -84826,7 +84414,7 @@
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>5540</v>
+        <v>5515</v>
       </c>
       <c r="J42" t="n">
         <v>1015</v>
@@ -85949,7 +85537,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2510</v>
+        <v>2525</v>
       </c>
       <c r="C64" t="n">
         <v>1165</v>
@@ -85970,7 +85558,7 @@
         <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>4650</v>
+        <v>4635</v>
       </c>
       <c r="J64" t="n">
         <v>1725</v>
@@ -86937,7 +86525,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>2355</v>
+        <v>2375</v>
       </c>
       <c r="C83" t="n">
         <v>2095</v>
@@ -86958,7 +86546,7 @@
         <v>0</v>
       </c>
       <c r="I83" t="n">
-        <v>4755</v>
+        <v>4735</v>
       </c>
       <c r="J83" t="n">
         <v>2140</v>
@@ -87613,7 +87201,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>3088</v>
+        <v>3108</v>
       </c>
       <c r="C96" t="n">
         <v>2384</v>
@@ -87634,7 +87222,7 @@
         <v>0</v>
       </c>
       <c r="I96" t="n">
-        <v>8656</v>
+        <v>8636</v>
       </c>
       <c r="J96" t="n">
         <v>2140</v>
@@ -88809,7 +88397,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>4468</v>
+        <v>4478</v>
       </c>
       <c r="C119" t="n">
         <v>1554</v>
@@ -88830,7 +88418,7 @@
         <v>0</v>
       </c>
       <c r="I119" t="n">
-        <v>9635</v>
+        <v>9625</v>
       </c>
       <c r="J119" t="n">
         <v>1110</v>
@@ -89797,7 +89385,7 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>3220</v>
+        <v>3222</v>
       </c>
       <c r="C138" t="n">
         <v>2564</v>
@@ -89818,7 +89406,7 @@
         <v>0</v>
       </c>
       <c r="I138" t="n">
-        <v>7872</v>
+        <v>7870</v>
       </c>
       <c r="J138" t="n">
         <v>1720</v>
@@ -89849,10 +89437,10 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>4164</v>
+        <v>4514</v>
       </c>
       <c r="C139" t="n">
-        <v>780</v>
+        <v>915</v>
       </c>
       <c r="D139" t="n">
         <v>385</v>
@@ -89870,10 +89458,10 @@
         <v>0</v>
       </c>
       <c r="I139" t="n">
-        <v>14578</v>
+        <v>16263</v>
       </c>
       <c r="J139" t="n">
-        <v>795</v>
+        <v>1610</v>
       </c>
       <c r="K139" t="n">
         <v>0</v>
@@ -89882,7 +89470,7 @@
         <v>425</v>
       </c>
       <c r="M139" t="n">
-        <v>0</v>
+        <v>745</v>
       </c>
       <c r="N139" t="n">
         <v>405</v>
@@ -89891,7 +89479,7 @@
         <v>690</v>
       </c>
       <c r="P139" t="n">
-        <v>22927</v>
+        <v>26657</v>
       </c>
     </row>
     <row r="140">
@@ -89901,10 +89489,10 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>396026</v>
+        <v>396508</v>
       </c>
       <c r="C140" t="n">
-        <v>221351</v>
+        <v>221486</v>
       </c>
       <c r="D140" t="n">
         <v>58168</v>
@@ -89922,10 +89510,10 @@
         <v>6860</v>
       </c>
       <c r="I140" t="n">
-        <v>741698</v>
+        <v>743251</v>
       </c>
       <c r="J140" t="n">
-        <v>217038</v>
+        <v>217853</v>
       </c>
       <c r="K140" t="n">
         <v>32660</v>
@@ -89934,7 +89522,7 @@
         <v>61344</v>
       </c>
       <c r="M140" t="n">
-        <v>99229</v>
+        <v>99974</v>
       </c>
       <c r="N140" t="n">
         <v>70576</v>
@@ -89943,7 +89531,7 @@
         <v>48134</v>
       </c>
       <c r="P140" t="n">
-        <v>2058792</v>
+        <v>2062522</v>
       </c>
     </row>
   </sheetData>
@@ -91349,7 +90937,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>780</v>
+        <v>915</v>
       </c>
     </row>
     <row r="140">
@@ -91359,7 +90947,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>221351</v>
+        <v>221486</v>
       </c>
     </row>
     <row r="142">
@@ -91467,7 +91055,7 @@
         <v>2026</v>
       </c>
       <c r="B154" t="n">
-        <v>12326</v>
+        <v>12461</v>
       </c>
     </row>
     <row r="155">
@@ -91477,7 +91065,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>221351</v>
+        <v>221486</v>
       </c>
     </row>
   </sheetData>
@@ -91563,7 +91151,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1581</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="8">
@@ -91623,7 +91211,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2077</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="14">
@@ -91913,7 +91501,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3363</v>
+        <v>3388</v>
       </c>
     </row>
     <row r="43">
@@ -92133,7 +91721,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2510</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="65">
@@ -92323,7 +91911,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>2355</v>
+        <v>2375</v>
       </c>
     </row>
     <row r="84">
@@ -92453,7 +92041,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>3088</v>
+        <v>3108</v>
       </c>
     </row>
     <row r="97">
@@ -92683,7 +92271,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>4468</v>
+        <v>4478</v>
       </c>
     </row>
     <row r="120">
@@ -92873,7 +92461,7 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>3220</v>
+        <v>3222</v>
       </c>
     </row>
     <row r="139">
@@ -92883,7 +92471,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>4164</v>
+        <v>4514</v>
       </c>
     </row>
     <row r="140">
@@ -92893,7 +92481,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>396026</v>
+        <v>396508</v>
       </c>
     </row>
     <row r="142">
@@ -92913,7 +92501,7 @@
         <v>2015</v>
       </c>
       <c r="B143" t="n">
-        <v>21247</v>
+        <v>21287</v>
       </c>
     </row>
     <row r="144">
@@ -92937,7 +92525,7 @@
         <v>2018</v>
       </c>
       <c r="B146" t="n">
-        <v>41697</v>
+        <v>41722</v>
       </c>
     </row>
     <row r="147">
@@ -92953,7 +92541,7 @@
         <v>2020</v>
       </c>
       <c r="B148" t="n">
-        <v>23257</v>
+        <v>23272</v>
       </c>
     </row>
     <row r="149">
@@ -92961,7 +92549,7 @@
         <v>2021</v>
       </c>
       <c r="B149" t="n">
-        <v>26144</v>
+        <v>26164</v>
       </c>
     </row>
     <row r="150">
@@ -92969,7 +92557,7 @@
         <v>2022</v>
       </c>
       <c r="B150" t="n">
-        <v>34219</v>
+        <v>34239</v>
       </c>
     </row>
     <row r="151">
@@ -92985,7 +92573,7 @@
         <v>2024</v>
       </c>
       <c r="B152" t="n">
-        <v>39604</v>
+        <v>39614</v>
       </c>
     </row>
     <row r="153">
@@ -93001,7 +92589,7 @@
         <v>2026</v>
       </c>
       <c r="B154" t="n">
-        <v>20805</v>
+        <v>21157</v>
       </c>
     </row>
     <row r="155">
@@ -93011,7 +92599,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>396026</v>
+        <v>396508</v>
       </c>
     </row>
   </sheetData>
@@ -93025,7 +92613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DX14"/>
+  <dimension ref="A1:DW14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -93661,11 +93249,6 @@
       </c>
       <c r="DW1" t="inlineStr">
         <is>
-          <t>Worcester</t>
-        </is>
-      </c>
-      <c r="DX1" t="inlineStr">
-        <is>
           <t>ROW_TOTAL</t>
         </is>
       </c>
@@ -93723,7 +93306,7 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>21247</v>
+        <v>21287</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
@@ -94050,9 +93633,6 @@
         <v>1082</v>
       </c>
       <c r="DW2" t="n">
-        <v>40</v>
-      </c>
-      <c r="DX2" t="n">
         <v>56684</v>
       </c>
     </row>
@@ -94436,9 +94016,6 @@
         <v>1675</v>
       </c>
       <c r="DW3" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX3" t="n">
         <v>90368</v>
       </c>
     </row>
@@ -94822,9 +94399,6 @@
         <v>2250</v>
       </c>
       <c r="DW4" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX4" t="n">
         <v>115971</v>
       </c>
     </row>
@@ -94881,7 +94455,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>45252</v>
+        <v>45277</v>
       </c>
       <c r="S5" t="n">
         <v>175</v>
@@ -95208,9 +94782,6 @@
         <v>2855</v>
       </c>
       <c r="DW5" t="n">
-        <v>25</v>
-      </c>
-      <c r="DX5" t="n">
         <v>161333</v>
       </c>
     </row>
@@ -95594,9 +95165,6 @@
         <v>3245</v>
       </c>
       <c r="DW6" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX6" t="n">
         <v>176032</v>
       </c>
     </row>
@@ -95653,7 +95221,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>25877</v>
+        <v>25892</v>
       </c>
       <c r="S7" t="n">
         <v>75</v>
@@ -95980,9 +95548,6 @@
         <v>2095</v>
       </c>
       <c r="DW7" t="n">
-        <v>15</v>
-      </c>
-      <c r="DX7" t="n">
         <v>146561</v>
       </c>
     </row>
@@ -96039,7 +95604,7 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>28879</v>
+        <v>28899</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
@@ -96366,9 +95931,6 @@
         <v>1580</v>
       </c>
       <c r="DW8" t="n">
-        <v>20</v>
-      </c>
-      <c r="DX8" t="n">
         <v>167907</v>
       </c>
     </row>
@@ -96425,7 +95987,7 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>37809</v>
+        <v>37829</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
@@ -96752,9 +96314,6 @@
         <v>1755</v>
       </c>
       <c r="DW9" t="n">
-        <v>20</v>
-      </c>
-      <c r="DX9" t="n">
         <v>226389</v>
       </c>
     </row>
@@ -97138,9 +96697,6 @@
         <v>2597</v>
       </c>
       <c r="DW10" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX10" t="n">
         <v>244406</v>
       </c>
     </row>
@@ -97197,7 +96753,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>44579</v>
+        <v>44589</v>
       </c>
       <c r="S11" t="n">
         <v>85</v>
@@ -97524,9 +97080,6 @@
         <v>3700</v>
       </c>
       <c r="DW11" t="n">
-        <v>10</v>
-      </c>
-      <c r="DX11" t="n">
         <v>263335</v>
       </c>
     </row>
@@ -97910,9 +97463,6 @@
         <v>3034</v>
       </c>
       <c r="DW12" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX12" t="n">
         <v>269977</v>
       </c>
     </row>
@@ -97930,7 +97480,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>3950</v>
+        <v>4070</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -97969,7 +97519,7 @@
         <v>105</v>
       </c>
       <c r="R13" t="n">
-        <v>23250</v>
+        <v>23602</v>
       </c>
       <c r="S13" t="n">
         <v>140</v>
@@ -97987,7 +97537,7 @@
         <v>1960</v>
       </c>
       <c r="X13" t="n">
-        <v>550</v>
+        <v>720</v>
       </c>
       <c r="Y13" t="n">
         <v>95</v>
@@ -97999,7 +97549,7 @@
         <v>2</v>
       </c>
       <c r="AB13" t="n">
-        <v>665</v>
+        <v>815</v>
       </c>
       <c r="AC13" t="n">
         <v>210</v>
@@ -98032,7 +97582,7 @@
         <v>0</v>
       </c>
       <c r="AM13" t="n">
-        <v>2051</v>
+        <v>2116</v>
       </c>
       <c r="AN13" t="n">
         <v>165</v>
@@ -98104,7 +97654,7 @@
         <v>320</v>
       </c>
       <c r="BK13" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="BL13" t="n">
         <v>2541</v>
@@ -98122,7 +97672,7 @@
         <v>335</v>
       </c>
       <c r="BQ13" t="n">
-        <v>4942</v>
+        <v>4957</v>
       </c>
       <c r="BR13" t="n">
         <v>1510</v>
@@ -98161,10 +97711,10 @@
         <v>0</v>
       </c>
       <c r="CD13" t="n">
-        <v>1537</v>
+        <v>1635</v>
       </c>
       <c r="CE13" t="n">
-        <v>714</v>
+        <v>856</v>
       </c>
       <c r="CF13" t="n">
         <v>30</v>
@@ -98203,13 +97753,13 @@
         <v>0</v>
       </c>
       <c r="CR13" t="n">
-        <v>470</v>
+        <v>500</v>
       </c>
       <c r="CS13" t="n">
         <v>2</v>
       </c>
       <c r="CT13" t="n">
-        <v>4045</v>
+        <v>4375</v>
       </c>
       <c r="CU13" t="n">
         <v>925</v>
@@ -98221,25 +97771,25 @@
         <v>80</v>
       </c>
       <c r="CX13" t="n">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="CY13" t="n">
         <v>190</v>
       </c>
       <c r="CZ13" t="n">
-        <v>1860</v>
+        <v>2190</v>
       </c>
       <c r="DA13" t="n">
-        <v>860</v>
+        <v>910</v>
       </c>
       <c r="DB13" t="n">
-        <v>12965</v>
+        <v>13780</v>
       </c>
       <c r="DC13" t="n">
         <v>30</v>
       </c>
       <c r="DD13" t="n">
-        <v>83</v>
+        <v>153</v>
       </c>
       <c r="DE13" t="n">
         <v>0</v>
@@ -98257,7 +97807,7 @@
         <v>2195</v>
       </c>
       <c r="DJ13" t="n">
-        <v>4720</v>
+        <v>5465</v>
       </c>
       <c r="DK13" t="n">
         <v>420</v>
@@ -98281,7 +97831,7 @@
         <v>395</v>
       </c>
       <c r="DR13" t="n">
-        <v>4223</v>
+        <v>4446</v>
       </c>
       <c r="DS13" t="n">
         <v>0</v>
@@ -98296,10 +97846,7 @@
         <v>1470</v>
       </c>
       <c r="DW13" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX13" t="n">
-        <v>139829</v>
+        <v>143559</v>
       </c>
     </row>
     <row r="14">
@@ -98318,7 +97865,7 @@
         <v>150</v>
       </c>
       <c r="E14" t="n">
-        <v>71345</v>
+        <v>71465</v>
       </c>
       <c r="F14" t="n">
         <v>500</v>
@@ -98357,7 +97904,7 @@
         <v>107</v>
       </c>
       <c r="R14" t="n">
-        <v>428686</v>
+        <v>429168</v>
       </c>
       <c r="S14" t="n">
         <v>925</v>
@@ -98375,7 +97922,7 @@
         <v>23953</v>
       </c>
       <c r="X14" t="n">
-        <v>4542</v>
+        <v>4712</v>
       </c>
       <c r="Y14" t="n">
         <v>2947</v>
@@ -98387,7 +97934,7 @@
         <v>2</v>
       </c>
       <c r="AB14" t="n">
-        <v>8979</v>
+        <v>9129</v>
       </c>
       <c r="AC14" t="n">
         <v>212</v>
@@ -98420,7 +97967,7 @@
         <v>374</v>
       </c>
       <c r="AM14" t="n">
-        <v>50594</v>
+        <v>50659</v>
       </c>
       <c r="AN14" t="n">
         <v>4755</v>
@@ -98492,7 +98039,7 @@
         <v>1007</v>
       </c>
       <c r="BK14" t="n">
-        <v>650</v>
+        <v>660</v>
       </c>
       <c r="BL14" t="n">
         <v>47345</v>
@@ -98510,7 +98057,7 @@
         <v>7365</v>
       </c>
       <c r="BQ14" t="n">
-        <v>94080</v>
+        <v>94095</v>
       </c>
       <c r="BR14" t="n">
         <v>22072</v>
@@ -98549,10 +98096,10 @@
         <v>435</v>
       </c>
       <c r="CD14" t="n">
-        <v>15275</v>
+        <v>15373</v>
       </c>
       <c r="CE14" t="n">
-        <v>5629</v>
+        <v>5771</v>
       </c>
       <c r="CF14" t="n">
         <v>145</v>
@@ -98591,13 +98138,13 @@
         <v>277</v>
       </c>
       <c r="CR14" t="n">
-        <v>11874</v>
+        <v>11904</v>
       </c>
       <c r="CS14" t="n">
         <v>2</v>
       </c>
       <c r="CT14" t="n">
-        <v>64775</v>
+        <v>65105</v>
       </c>
       <c r="CU14" t="n">
         <v>2384</v>
@@ -98609,25 +98156,25 @@
         <v>2698</v>
       </c>
       <c r="CX14" t="n">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="CY14" t="n">
         <v>8936</v>
       </c>
       <c r="CZ14" t="n">
-        <v>18166</v>
+        <v>18496</v>
       </c>
       <c r="DA14" t="n">
-        <v>13716</v>
+        <v>13766</v>
       </c>
       <c r="DB14" t="n">
-        <v>217038</v>
+        <v>217853</v>
       </c>
       <c r="DC14" t="n">
         <v>1030</v>
       </c>
       <c r="DD14" t="n">
-        <v>1281</v>
+        <v>1351</v>
       </c>
       <c r="DE14" t="n">
         <v>1485</v>
@@ -98645,7 +98192,7 @@
         <v>23863</v>
       </c>
       <c r="DJ14" t="n">
-        <v>99229</v>
+        <v>99974</v>
       </c>
       <c r="DK14" t="n">
         <v>1240</v>
@@ -98669,7 +98216,7 @@
         <v>7725</v>
       </c>
       <c r="DR14" t="n">
-        <v>57518</v>
+        <v>57741</v>
       </c>
       <c r="DS14" t="n">
         <v>1450</v>
@@ -98684,10 +98231,7 @@
         <v>27338</v>
       </c>
       <c r="DW14" t="n">
-        <v>130</v>
-      </c>
-      <c r="DX14" t="n">
-        <v>2058792</v>
+        <v>2062522</v>
       </c>
     </row>
   </sheetData>
@@ -98815,7 +98359,7 @@
         <v>840</v>
       </c>
       <c r="E2" t="n">
-        <v>25851</v>
+        <v>25891</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -98848,7 +98392,7 @@
         <v>327</v>
       </c>
       <c r="P2" t="n">
-        <v>12980</v>
+        <v>12940</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -98992,7 +98536,7 @@
         <v>4090</v>
       </c>
       <c r="E5" t="n">
-        <v>71642</v>
+        <v>71667</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -99025,7 +98569,7 @@
         <v>1915</v>
       </c>
       <c r="P5" t="n">
-        <v>38452</v>
+        <v>38427</v>
       </c>
       <c r="Q5" t="n">
         <v>2850</v>
@@ -99110,7 +98654,7 @@
         <v>7463</v>
       </c>
       <c r="E7" t="n">
-        <v>57878</v>
+        <v>57893</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -99143,7 +98687,7 @@
         <v>1455</v>
       </c>
       <c r="P7" t="n">
-        <v>29055</v>
+        <v>29040</v>
       </c>
       <c r="Q7" t="n">
         <v>2250</v>
@@ -99169,7 +98713,7 @@
         <v>5949</v>
       </c>
       <c r="E8" t="n">
-        <v>64998</v>
+        <v>65018</v>
       </c>
       <c r="F8" t="n">
         <v>1141</v>
@@ -99187,13 +98731,13 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>7521</v>
+        <v>7266</v>
       </c>
       <c r="L8" t="n">
         <v>3015</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>255</v>
       </c>
       <c r="N8" t="n">
         <v>25</v>
@@ -99202,7 +98746,7 @@
         <v>1090</v>
       </c>
       <c r="P8" t="n">
-        <v>35089</v>
+        <v>35069</v>
       </c>
       <c r="Q8" t="n">
         <v>3365</v>
@@ -99228,7 +98772,7 @@
         <v>8150</v>
       </c>
       <c r="E9" t="n">
-        <v>95265</v>
+        <v>95285</v>
       </c>
       <c r="F9" t="n">
         <v>1875</v>
@@ -99246,13 +98790,13 @@
         <v>94</v>
       </c>
       <c r="K9" t="n">
-        <v>10425</v>
+        <v>9985</v>
       </c>
       <c r="L9" t="n">
         <v>3855</v>
       </c>
       <c r="M9" t="n">
-        <v>618</v>
+        <v>1058</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -99261,7 +98805,7 @@
         <v>3273</v>
       </c>
       <c r="P9" t="n">
-        <v>40897</v>
+        <v>40877</v>
       </c>
       <c r="Q9" t="n">
         <v>4700</v>
@@ -99305,13 +98849,13 @@
         <v>498</v>
       </c>
       <c r="K10" t="n">
-        <v>12017</v>
+        <v>11600</v>
       </c>
       <c r="L10" t="n">
         <v>3155</v>
       </c>
       <c r="M10" t="n">
-        <v>1039</v>
+        <v>1456</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -99346,7 +98890,7 @@
         <v>8374</v>
       </c>
       <c r="E11" t="n">
-        <v>104799</v>
+        <v>104809</v>
       </c>
       <c r="F11" t="n">
         <v>714</v>
@@ -99364,13 +98908,13 @@
         <v>1970</v>
       </c>
       <c r="K11" t="n">
-        <v>13887</v>
+        <v>13417</v>
       </c>
       <c r="L11" t="n">
         <v>5151</v>
       </c>
       <c r="M11" t="n">
-        <v>1429</v>
+        <v>1899</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -99379,7 +98923,7 @@
         <v>2692</v>
       </c>
       <c r="P11" t="n">
-        <v>50534</v>
+        <v>50524</v>
       </c>
       <c r="Q11" t="n">
         <v>6476</v>
@@ -99423,13 +98967,13 @@
         <v>1465</v>
       </c>
       <c r="K12" t="n">
-        <v>17019</v>
+        <v>16399</v>
       </c>
       <c r="L12" t="n">
         <v>3284</v>
       </c>
       <c r="M12" t="n">
-        <v>1829</v>
+        <v>2449</v>
       </c>
       <c r="N12" t="n">
         <v>17</v>
@@ -99461,34 +99005,34 @@
         <v>2075</v>
       </c>
       <c r="D13" t="n">
-        <v>4400</v>
+        <v>4780</v>
       </c>
       <c r="E13" t="n">
-        <v>58520</v>
+        <v>59520</v>
       </c>
       <c r="F13" t="n">
         <v>465</v>
       </c>
       <c r="G13" t="n">
-        <v>2410</v>
+        <v>2825</v>
       </c>
       <c r="H13" t="n">
         <v>1215</v>
       </c>
       <c r="I13" t="n">
-        <v>17431</v>
+        <v>18246</v>
       </c>
       <c r="J13" t="n">
         <v>912</v>
       </c>
       <c r="K13" t="n">
-        <v>8943</v>
+        <v>8763</v>
       </c>
       <c r="L13" t="n">
         <v>2177</v>
       </c>
       <c r="M13" t="n">
-        <v>714</v>
+        <v>1036</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -99497,7 +99041,7 @@
         <v>200</v>
       </c>
       <c r="P13" t="n">
-        <v>24365</v>
+        <v>25343</v>
       </c>
       <c r="Q13" t="n">
         <v>3227</v>
@@ -99506,7 +99050,7 @@
         <v>8112</v>
       </c>
       <c r="S13" t="n">
-        <v>139829</v>
+        <v>143559</v>
       </c>
     </row>
     <row r="14">
@@ -99522,34 +99066,34 @@
         <v>17331</v>
       </c>
       <c r="D14" t="n">
-        <v>61678</v>
+        <v>62058</v>
       </c>
       <c r="E14" t="n">
-        <v>850112</v>
+        <v>851242</v>
       </c>
       <c r="F14" t="n">
         <v>5932</v>
       </c>
       <c r="G14" t="n">
-        <v>33600</v>
+        <v>34015</v>
       </c>
       <c r="H14" t="n">
         <v>7499</v>
       </c>
       <c r="I14" t="n">
-        <v>282329</v>
+        <v>283144</v>
       </c>
       <c r="J14" t="n">
         <v>4939</v>
       </c>
       <c r="K14" t="n">
-        <v>111442</v>
+        <v>109060</v>
       </c>
       <c r="L14" t="n">
         <v>35385</v>
       </c>
       <c r="M14" t="n">
-        <v>5629</v>
+        <v>8153</v>
       </c>
       <c r="N14" t="n">
         <v>42</v>
@@ -99558,7 +99102,7 @@
         <v>22052</v>
       </c>
       <c r="P14" t="n">
-        <v>419016</v>
+        <v>419864</v>
       </c>
       <c r="Q14" t="n">
         <v>36635</v>
@@ -99567,7 +99111,7 @@
         <v>87453</v>
       </c>
       <c r="S14" t="n">
-        <v>2058792</v>
+        <v>2062522</v>
       </c>
     </row>
   </sheetData>
@@ -99671,7 +99215,7 @@
         <v>2015</v>
       </c>
       <c r="B2" t="n">
-        <v>21247</v>
+        <v>21287</v>
       </c>
       <c r="C2" t="n">
         <v>6670</v>
@@ -99692,7 +99236,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>8126</v>
+        <v>8086</v>
       </c>
       <c r="J2" t="n">
         <v>6885</v>
@@ -99821,7 +99365,7 @@
         <v>2018</v>
       </c>
       <c r="B5" t="n">
-        <v>41697</v>
+        <v>41722</v>
       </c>
       <c r="C5" t="n">
         <v>21112</v>
@@ -99842,7 +99386,7 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>43656</v>
+        <v>43631</v>
       </c>
       <c r="J5" t="n">
         <v>13913</v>
@@ -99921,7 +99465,7 @@
         <v>2020</v>
       </c>
       <c r="B7" t="n">
-        <v>23257</v>
+        <v>23272</v>
       </c>
       <c r="C7" t="n">
         <v>15805</v>
@@ -99942,7 +99486,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>56553</v>
+        <v>56538</v>
       </c>
       <c r="J7" t="n">
         <v>17285</v>
@@ -99971,7 +99515,7 @@
         <v>2021</v>
       </c>
       <c r="B8" t="n">
-        <v>26144</v>
+        <v>26164</v>
       </c>
       <c r="C8" t="n">
         <v>18542</v>
@@ -99992,7 +99536,7 @@
         <v>825</v>
       </c>
       <c r="I8" t="n">
-        <v>65041</v>
+        <v>65021</v>
       </c>
       <c r="J8" t="n">
         <v>21884</v>
@@ -100021,7 +99565,7 @@
         <v>2022</v>
       </c>
       <c r="B9" t="n">
-        <v>34219</v>
+        <v>34239</v>
       </c>
       <c r="C9" t="n">
         <v>22238</v>
@@ -100042,7 +99586,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>101046</v>
+        <v>101026</v>
       </c>
       <c r="J9" t="n">
         <v>25698</v>
@@ -100121,7 +99665,7 @@
         <v>2024</v>
       </c>
       <c r="B11" t="n">
-        <v>39604</v>
+        <v>39614</v>
       </c>
       <c r="C11" t="n">
         <v>27438</v>
@@ -100142,7 +99686,7 @@
         <v>95</v>
       </c>
       <c r="I11" t="n">
-        <v>105075</v>
+        <v>105065</v>
       </c>
       <c r="J11" t="n">
         <v>26942</v>
@@ -100221,10 +99765,10 @@
         <v>2026</v>
       </c>
       <c r="B13" t="n">
-        <v>20805</v>
+        <v>21157</v>
       </c>
       <c r="C13" t="n">
-        <v>12326</v>
+        <v>12461</v>
       </c>
       <c r="D13" t="n">
         <v>4107</v>
@@ -100242,10 +99786,10 @@
         <v>2690</v>
       </c>
       <c r="I13" t="n">
-        <v>58695</v>
+        <v>60378</v>
       </c>
       <c r="J13" t="n">
-        <v>12965</v>
+        <v>13780</v>
       </c>
       <c r="K13" t="n">
         <v>2445</v>
@@ -100254,7 +99798,7 @@
         <v>5000</v>
       </c>
       <c r="M13" t="n">
-        <v>4720</v>
+        <v>5465</v>
       </c>
       <c r="N13" t="n">
         <v>4790</v>
@@ -100263,7 +99807,7 @@
         <v>3160</v>
       </c>
       <c r="P13" t="n">
-        <v>139829</v>
+        <v>143559</v>
       </c>
     </row>
     <row r="14">
@@ -100273,10 +99817,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>396026</v>
+        <v>396508</v>
       </c>
       <c r="C14" t="n">
-        <v>221351</v>
+        <v>221486</v>
       </c>
       <c r="D14" t="n">
         <v>58168</v>
@@ -100294,10 +99838,10 @@
         <v>6860</v>
       </c>
       <c r="I14" t="n">
-        <v>741698</v>
+        <v>743251</v>
       </c>
       <c r="J14" t="n">
-        <v>217038</v>
+        <v>217853</v>
       </c>
       <c r="K14" t="n">
         <v>32660</v>
@@ -100306,7 +99850,7 @@
         <v>61344</v>
       </c>
       <c r="M14" t="n">
-        <v>99229</v>
+        <v>99974</v>
       </c>
       <c r="N14" t="n">
         <v>70576</v>
@@ -100315,7 +99859,7 @@
         <v>48134</v>
       </c>
       <c r="P14" t="n">
-        <v>2058792</v>
+        <v>2062522</v>
       </c>
     </row>
   </sheetData>
@@ -100697,10 +100241,10 @@
         <v>830</v>
       </c>
       <c r="N7" t="n">
-        <v>1581</v>
+        <v>1606</v>
       </c>
       <c r="O7" t="n">
-        <v>3653</v>
+        <v>3678</v>
       </c>
     </row>
     <row r="8">
@@ -100991,10 +100535,10 @@
         <v>482</v>
       </c>
       <c r="N13" t="n">
-        <v>2077</v>
+        <v>2092</v>
       </c>
       <c r="O13" t="n">
-        <v>4513</v>
+        <v>4528</v>
       </c>
     </row>
     <row r="14">
@@ -101040,10 +100584,10 @@
         <v>6670</v>
       </c>
       <c r="N14" t="n">
-        <v>21247</v>
+        <v>21287</v>
       </c>
       <c r="O14" t="n">
-        <v>48558</v>
+        <v>48598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 2 data contract validation and cache busting
</commit_message>
<xml_diff>
--- a/oil_collection_report.xlsx
+++ b/oil_collection_report.xlsx
@@ -53415,7 +53415,7 @@
         <v>0</v>
       </c>
       <c r="M140" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="N140" t="n">
         <v>0</v>
@@ -53430,7 +53430,7 @@
         <v>0</v>
       </c>
       <c r="R140" t="n">
-        <v>3435</v>
+        <v>3710</v>
       </c>
       <c r="S140" t="n">
         <v>50</v>
@@ -53445,7 +53445,7 @@
         <v>0</v>
       </c>
       <c r="W140" t="n">
-        <v>410</v>
+        <v>460</v>
       </c>
       <c r="X140" t="n">
         <v>110</v>
@@ -53490,13 +53490,13 @@
         <v>55</v>
       </c>
       <c r="AL140" t="n">
-        <v>75</v>
+        <v>746</v>
       </c>
       <c r="AM140" t="n">
         <v>0</v>
       </c>
       <c r="AN140" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="AO140" t="n">
         <v>7</v>
@@ -53508,7 +53508,7 @@
         <v>0</v>
       </c>
       <c r="AR140" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AS140" t="n">
         <v>275</v>
@@ -53529,7 +53529,7 @@
         <v>0</v>
       </c>
       <c r="AY140" t="n">
-        <v>290</v>
+        <v>370</v>
       </c>
       <c r="AZ140" t="n">
         <v>0</v>
@@ -53589,13 +53589,13 @@
         <v>0</v>
       </c>
       <c r="BS140" t="n">
-        <v>420</v>
+        <v>950</v>
       </c>
       <c r="BT140" t="n">
         <v>305</v>
       </c>
       <c r="BU140" t="n">
-        <v>0</v>
+        <v>505</v>
       </c>
       <c r="BV140" t="n">
         <v>455</v>
@@ -53721,7 +53721,7 @@
         <v>0</v>
       </c>
       <c r="DK140" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="DL140" t="n">
         <v>251</v>
@@ -53742,7 +53742,7 @@
         <v>0</v>
       </c>
       <c r="DR140" t="n">
-        <v>755</v>
+        <v>995</v>
       </c>
       <c r="DS140" t="n">
         <v>0</v>
@@ -53751,7 +53751,7 @@
         <v>70</v>
       </c>
       <c r="DU140" t="n">
-        <v>19983</v>
+        <v>23104</v>
       </c>
     </row>
     <row r="141">
@@ -53794,7 +53794,7 @@
         <v>5790</v>
       </c>
       <c r="M141" t="n">
-        <v>1582</v>
+        <v>1742</v>
       </c>
       <c r="N141" t="n">
         <v>2935</v>
@@ -53809,7 +53809,7 @@
         <v>105</v>
       </c>
       <c r="R141" t="n">
-        <v>432768</v>
+        <v>433043</v>
       </c>
       <c r="S141" t="n">
         <v>975</v>
@@ -53824,7 +53824,7 @@
         <v>14436</v>
       </c>
       <c r="W141" t="n">
-        <v>24359</v>
+        <v>24409</v>
       </c>
       <c r="X141" t="n">
         <v>4820</v>
@@ -53869,13 +53869,13 @@
         <v>427</v>
       </c>
       <c r="AL141" t="n">
-        <v>50732</v>
+        <v>51403</v>
       </c>
       <c r="AM141" t="n">
         <v>4755</v>
       </c>
       <c r="AN141" t="n">
-        <v>3355</v>
+        <v>3715</v>
       </c>
       <c r="AO141" t="n">
         <v>282</v>
@@ -53887,7 +53887,7 @@
         <v>385</v>
       </c>
       <c r="AR141" t="n">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="AS141" t="n">
         <v>26879</v>
@@ -53908,7 +53908,7 @@
         <v>460</v>
       </c>
       <c r="AY141" t="n">
-        <v>41222</v>
+        <v>41302</v>
       </c>
       <c r="AZ141" t="n">
         <v>6666</v>
@@ -53968,13 +53968,13 @@
         <v>13430</v>
       </c>
       <c r="BS141" t="n">
-        <v>26996</v>
+        <v>27526</v>
       </c>
       <c r="BT141" t="n">
         <v>5420</v>
       </c>
       <c r="BU141" t="n">
-        <v>5785</v>
+        <v>6290</v>
       </c>
       <c r="BV141" t="n">
         <v>34940</v>
@@ -54100,7 +54100,7 @@
         <v>15330</v>
       </c>
       <c r="DK141" t="n">
-        <v>10550</v>
+        <v>10780</v>
       </c>
       <c r="DL141" t="n">
         <v>18216</v>
@@ -54121,7 +54121,7 @@
         <v>1450</v>
       </c>
       <c r="DR141" t="n">
-        <v>71327</v>
+        <v>71567</v>
       </c>
       <c r="DS141" t="n">
         <v>4927</v>
@@ -54130,7 +54130,7 @@
         <v>27596</v>
       </c>
       <c r="DU141" t="n">
-        <v>2089759</v>
+        <v>2092880</v>
       </c>
     </row>
   </sheetData>
@@ -60361,10 +60361,10 @@
         <v>915</v>
       </c>
       <c r="F8" t="n">
-        <v>425</v>
+        <v>1010</v>
       </c>
       <c r="G8" t="n">
-        <v>755</v>
+        <v>995</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -60385,10 +60385,10 @@
         <v>1810</v>
       </c>
       <c r="N8" t="n">
-        <v>3435</v>
+        <v>3710</v>
       </c>
       <c r="O8" t="n">
-        <v>12125</v>
+        <v>13225</v>
       </c>
     </row>
     <row r="9">
@@ -60410,10 +60410,10 @@
         <v>4521</v>
       </c>
       <c r="F9" t="n">
-        <v>4530</v>
+        <v>5115</v>
       </c>
       <c r="G9" t="n">
-        <v>5545</v>
+        <v>5785</v>
       </c>
       <c r="H9" t="n">
         <v>2445</v>
@@ -60434,10 +60434,10 @@
         <v>15989</v>
       </c>
       <c r="N9" t="n">
-        <v>24797</v>
+        <v>25072</v>
       </c>
       <c r="O9" t="n">
-        <v>97772</v>
+        <v>98872</v>
       </c>
     </row>
   </sheetData>
@@ -63657,7 +63657,7 @@
         <v>390</v>
       </c>
       <c r="L27" t="n">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -63666,7 +63666,7 @@
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>460</v>
+        <v>475</v>
       </c>
       <c r="P27" t="n">
         <v>2007</v>
@@ -63840,7 +63840,7 @@
         <v>270</v>
       </c>
       <c r="L30" t="n">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
@@ -63849,7 +63849,7 @@
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="P30" t="n">
         <v>2738</v>
@@ -63962,7 +63962,7 @@
         <v>1280</v>
       </c>
       <c r="L32" t="n">
-        <v>220</v>
+        <v>170</v>
       </c>
       <c r="M32" t="n">
         <v>0</v>
@@ -63971,7 +63971,7 @@
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>145</v>
+        <v>195</v>
       </c>
       <c r="P32" t="n">
         <v>2590</v>
@@ -64023,7 +64023,7 @@
         <v>325</v>
       </c>
       <c r="L33" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="M33" t="n">
         <v>0</v>
@@ -64032,7 +64032,7 @@
         <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>240</v>
+        <v>290</v>
       </c>
       <c r="P33" t="n">
         <v>2630</v>
@@ -64084,7 +64084,7 @@
         <v>720</v>
       </c>
       <c r="L34" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="M34" t="n">
         <v>0</v>
@@ -64093,7 +64093,7 @@
         <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="P34" t="n">
         <v>4360</v>
@@ -64206,7 +64206,7 @@
         <v>385</v>
       </c>
       <c r="L36" t="n">
-        <v>500</v>
+        <v>440</v>
       </c>
       <c r="M36" t="n">
         <v>0</v>
@@ -64215,7 +64215,7 @@
         <v>0</v>
       </c>
       <c r="O36" t="n">
-        <v>340</v>
+        <v>400</v>
       </c>
       <c r="P36" t="n">
         <v>2225</v>
@@ -64328,7 +64328,7 @@
         <v>250</v>
       </c>
       <c r="L38" t="n">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="M38" t="n">
         <v>0</v>
@@ -64337,7 +64337,7 @@
         <v>0</v>
       </c>
       <c r="O38" t="n">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="P38" t="n">
         <v>2295</v>
@@ -64572,7 +64572,7 @@
         <v>550</v>
       </c>
       <c r="L42" t="n">
-        <v>250</v>
+        <v>75</v>
       </c>
       <c r="M42" t="n">
         <v>0</v>
@@ -64581,7 +64581,7 @@
         <v>0</v>
       </c>
       <c r="O42" t="n">
-        <v>275</v>
+        <v>450</v>
       </c>
       <c r="P42" t="n">
         <v>2492</v>
@@ -64755,7 +64755,7 @@
         <v>1410</v>
       </c>
       <c r="L45" t="n">
-        <v>425</v>
+        <v>250</v>
       </c>
       <c r="M45" t="n">
         <v>0</v>
@@ -64764,7 +64764,7 @@
         <v>0</v>
       </c>
       <c r="O45" t="n">
-        <v>50</v>
+        <v>225</v>
       </c>
       <c r="P45" t="n">
         <v>3217</v>
@@ -64877,7 +64877,7 @@
         <v>1050</v>
       </c>
       <c r="L47" t="n">
-        <v>245</v>
+        <v>185</v>
       </c>
       <c r="M47" t="n">
         <v>0</v>
@@ -64886,7 +64886,7 @@
         <v>0</v>
       </c>
       <c r="O47" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="P47" t="n">
         <v>3385</v>
@@ -65182,7 +65182,7 @@
         <v>1010</v>
       </c>
       <c r="L52" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="M52" t="n">
         <v>0</v>
@@ -65191,7 +65191,7 @@
         <v>0</v>
       </c>
       <c r="O52" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="P52" t="n">
         <v>3350</v>
@@ -65304,7 +65304,7 @@
         <v>935</v>
       </c>
       <c r="L54" t="n">
-        <v>645</v>
+        <v>600</v>
       </c>
       <c r="M54" t="n">
         <v>0</v>
@@ -65313,7 +65313,7 @@
         <v>0</v>
       </c>
       <c r="O54" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="P54" t="n">
         <v>3975</v>
@@ -65487,7 +65487,7 @@
         <v>60</v>
       </c>
       <c r="L57" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="M57" t="n">
         <v>0</v>
@@ -65496,7 +65496,7 @@
         <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="P57" t="n">
         <v>2925</v>
@@ -65792,16 +65792,16 @@
         <v>910</v>
       </c>
       <c r="L62" t="n">
+        <v>0</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
         <v>40</v>
-      </c>
-      <c r="M62" t="n">
-        <v>0</v>
-      </c>
-      <c r="N62" t="n">
-        <v>0</v>
-      </c>
-      <c r="O62" t="n">
-        <v>0</v>
       </c>
       <c r="P62" t="n">
         <v>2400</v>
@@ -65914,7 +65914,7 @@
         <v>75</v>
       </c>
       <c r="L64" t="n">
-        <v>400</v>
+        <v>275</v>
       </c>
       <c r="M64" t="n">
         <v>0</v>
@@ -65923,7 +65923,7 @@
         <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>165</v>
+        <v>290</v>
       </c>
       <c r="P64" t="n">
         <v>3335</v>
@@ -66097,7 +66097,7 @@
         <v>0</v>
       </c>
       <c r="L67" t="n">
-        <v>375</v>
+        <v>325</v>
       </c>
       <c r="M67" t="n">
         <v>0</v>
@@ -66106,7 +66106,7 @@
         <v>0</v>
       </c>
       <c r="O67" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P67" t="n">
         <v>2670</v>
@@ -66280,7 +66280,7 @@
         <v>550</v>
       </c>
       <c r="L70" t="n">
-        <v>595</v>
+        <v>475</v>
       </c>
       <c r="M70" t="n">
         <v>0</v>
@@ -66289,7 +66289,7 @@
         <v>0</v>
       </c>
       <c r="O70" t="n">
-        <v>250</v>
+        <v>370</v>
       </c>
       <c r="P70" t="n">
         <v>2985</v>
@@ -66402,7 +66402,7 @@
         <v>1015</v>
       </c>
       <c r="L72" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="M72" t="n">
         <v>0</v>
@@ -66411,7 +66411,7 @@
         <v>0</v>
       </c>
       <c r="O72" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="P72" t="n">
         <v>2865</v>
@@ -66524,7 +66524,7 @@
         <v>525</v>
       </c>
       <c r="L74" t="n">
-        <v>385</v>
+        <v>305</v>
       </c>
       <c r="M74" t="n">
         <v>0</v>
@@ -66533,7 +66533,7 @@
         <v>0</v>
       </c>
       <c r="O74" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="P74" t="n">
         <v>1985</v>
@@ -66768,7 +66768,7 @@
         <v>600</v>
       </c>
       <c r="L78" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="M78" t="n">
         <v>0</v>
@@ -66777,7 +66777,7 @@
         <v>0</v>
       </c>
       <c r="O78" t="n">
-        <v>175</v>
+        <v>325</v>
       </c>
       <c r="P78" t="n">
         <v>2225</v>
@@ -66951,7 +66951,7 @@
         <v>940</v>
       </c>
       <c r="L81" t="n">
-        <v>380</v>
+        <v>305</v>
       </c>
       <c r="M81" t="n">
         <v>0</v>
@@ -66960,7 +66960,7 @@
         <v>0</v>
       </c>
       <c r="O81" t="n">
-        <v>150</v>
+        <v>225</v>
       </c>
       <c r="P81" t="n">
         <v>3530</v>
@@ -67012,7 +67012,7 @@
         <v>0</v>
       </c>
       <c r="L82" t="n">
-        <v>305</v>
+        <v>285</v>
       </c>
       <c r="M82" t="n">
         <v>0</v>
@@ -67021,7 +67021,7 @@
         <v>0</v>
       </c>
       <c r="O82" t="n">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="P82" t="n">
         <v>3570</v>
@@ -67070,13 +67070,13 @@
         <v>0</v>
       </c>
       <c r="K83" t="n">
-        <v>990</v>
+        <v>1070</v>
       </c>
       <c r="L83" t="n">
         <v>205</v>
       </c>
       <c r="M83" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="N83" t="n">
         <v>0</v>
@@ -67131,13 +67131,13 @@
         <v>0</v>
       </c>
       <c r="K84" t="n">
-        <v>125</v>
+        <v>200</v>
       </c>
       <c r="L84" t="n">
         <v>155</v>
       </c>
       <c r="M84" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="N84" t="n">
         <v>0</v>
@@ -67192,19 +67192,19 @@
         <v>0</v>
       </c>
       <c r="K85" t="n">
-        <v>891</v>
+        <v>991</v>
       </c>
       <c r="L85" t="n">
-        <v>210</v>
+        <v>160</v>
       </c>
       <c r="M85" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="N85" t="n">
         <v>25</v>
       </c>
       <c r="O85" t="n">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="P85" t="n">
         <v>3740</v>
@@ -67314,13 +67314,13 @@
         <v>0</v>
       </c>
       <c r="K87" t="n">
-        <v>1395</v>
+        <v>1425</v>
       </c>
       <c r="L87" t="n">
         <v>260</v>
       </c>
       <c r="M87" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N87" t="n">
         <v>0</v>
@@ -67375,19 +67375,19 @@
         <v>0</v>
       </c>
       <c r="K88" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="L88" t="n">
-        <v>405</v>
+        <v>255</v>
       </c>
       <c r="M88" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="N88" t="n">
         <v>0</v>
       </c>
       <c r="O88" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="P88" t="n">
         <v>3779</v>
@@ -67436,13 +67436,13 @@
         <v>0</v>
       </c>
       <c r="K89" t="n">
-        <v>1920</v>
+        <v>2100</v>
       </c>
       <c r="L89" t="n">
         <v>210</v>
       </c>
       <c r="M89" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="N89" t="n">
         <v>0</v>
@@ -67497,13 +67497,13 @@
         <v>0</v>
       </c>
       <c r="K90" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="L90" t="n">
         <v>205</v>
       </c>
       <c r="M90" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="N90" t="n">
         <v>0</v>
@@ -67561,7 +67561,7 @@
         <v>1030</v>
       </c>
       <c r="L91" t="n">
-        <v>305</v>
+        <v>255</v>
       </c>
       <c r="M91" t="n">
         <v>0</v>
@@ -67570,7 +67570,7 @@
         <v>0</v>
       </c>
       <c r="O91" t="n">
-        <v>285</v>
+        <v>335</v>
       </c>
       <c r="P91" t="n">
         <v>3435</v>
@@ -67619,13 +67619,13 @@
         <v>0</v>
       </c>
       <c r="K92" t="n">
-        <v>453</v>
+        <v>493</v>
       </c>
       <c r="L92" t="n">
         <v>415</v>
       </c>
       <c r="M92" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="N92" t="n">
         <v>0</v>
@@ -67680,13 +67680,13 @@
         <v>0</v>
       </c>
       <c r="K93" t="n">
-        <v>1290</v>
+        <v>1360</v>
       </c>
       <c r="L93" t="n">
         <v>0</v>
       </c>
       <c r="M93" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="N93" t="n">
         <v>0</v>
@@ -67744,7 +67744,7 @@
         <v>1182</v>
       </c>
       <c r="L94" t="n">
-        <v>692</v>
+        <v>612</v>
       </c>
       <c r="M94" t="n">
         <v>385</v>
@@ -67753,7 +67753,7 @@
         <v>0</v>
       </c>
       <c r="O94" t="n">
-        <v>755</v>
+        <v>835</v>
       </c>
       <c r="P94" t="n">
         <v>4228</v>
@@ -67802,13 +67802,13 @@
         <v>0</v>
       </c>
       <c r="K95" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="L95" t="n">
         <v>367</v>
       </c>
       <c r="M95" t="n">
-        <v>166</v>
+        <v>126</v>
       </c>
       <c r="N95" t="n">
         <v>0</v>
@@ -67927,7 +67927,7 @@
         <v>778</v>
       </c>
       <c r="L97" t="n">
-        <v>394</v>
+        <v>319</v>
       </c>
       <c r="M97" t="n">
         <v>107</v>
@@ -67936,7 +67936,7 @@
         <v>0</v>
       </c>
       <c r="O97" t="n">
-        <v>470</v>
+        <v>545</v>
       </c>
       <c r="P97" t="n">
         <v>2444</v>
@@ -67985,13 +67985,13 @@
         <v>85</v>
       </c>
       <c r="K98" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="L98" t="n">
         <v>354</v>
       </c>
       <c r="M98" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="N98" t="n">
         <v>0</v>
@@ -68107,13 +68107,13 @@
         <v>0</v>
       </c>
       <c r="K100" t="n">
-        <v>925</v>
+        <v>975</v>
       </c>
       <c r="L100" t="n">
         <v>284</v>
       </c>
       <c r="M100" t="n">
-        <v>177</v>
+        <v>127</v>
       </c>
       <c r="N100" t="n">
         <v>0</v>
@@ -68171,7 +68171,7 @@
         <v>895</v>
       </c>
       <c r="L101" t="n">
-        <v>375</v>
+        <v>285</v>
       </c>
       <c r="M101" t="n">
         <v>0</v>
@@ -68180,7 +68180,7 @@
         <v>0</v>
       </c>
       <c r="O101" t="n">
-        <v>298</v>
+        <v>388</v>
       </c>
       <c r="P101" t="n">
         <v>3979</v>
@@ -68229,13 +68229,13 @@
         <v>75</v>
       </c>
       <c r="K102" t="n">
-        <v>675</v>
+        <v>745</v>
       </c>
       <c r="L102" t="n">
         <v>313</v>
       </c>
       <c r="M102" t="n">
-        <v>198</v>
+        <v>128</v>
       </c>
       <c r="N102" t="n">
         <v>0</v>
@@ -68290,19 +68290,19 @@
         <v>0</v>
       </c>
       <c r="K103" t="n">
-        <v>1780</v>
+        <v>1847</v>
       </c>
       <c r="L103" t="n">
-        <v>440</v>
+        <v>395</v>
       </c>
       <c r="M103" t="n">
-        <v>205</v>
+        <v>138</v>
       </c>
       <c r="N103" t="n">
         <v>0</v>
       </c>
       <c r="O103" t="n">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="P103" t="n">
         <v>5056</v>
@@ -68473,13 +68473,13 @@
         <v>163</v>
       </c>
       <c r="K106" t="n">
-        <v>762</v>
+        <v>862</v>
       </c>
       <c r="L106" t="n">
         <v>378</v>
       </c>
       <c r="M106" t="n">
-        <v>228</v>
+        <v>128</v>
       </c>
       <c r="N106" t="n">
         <v>0</v>
@@ -68537,7 +68537,7 @@
         <v>550</v>
       </c>
       <c r="L107" t="n">
-        <v>329</v>
+        <v>289</v>
       </c>
       <c r="M107" t="n">
         <v>143</v>
@@ -68546,7 +68546,7 @@
         <v>0</v>
       </c>
       <c r="O107" t="n">
-        <v>305</v>
+        <v>345</v>
       </c>
       <c r="P107" t="n">
         <v>4725</v>
@@ -68595,13 +68595,13 @@
         <v>0</v>
       </c>
       <c r="K108" t="n">
-        <v>955</v>
+        <v>1015</v>
       </c>
       <c r="L108" t="n">
         <v>439</v>
       </c>
       <c r="M108" t="n">
-        <v>197</v>
+        <v>137</v>
       </c>
       <c r="N108" t="n">
         <v>0</v>
@@ -68778,13 +68778,13 @@
         <v>45</v>
       </c>
       <c r="K111" t="n">
-        <v>1936</v>
+        <v>2026</v>
       </c>
       <c r="L111" t="n">
         <v>414</v>
       </c>
       <c r="M111" t="n">
-        <v>194</v>
+        <v>104</v>
       </c>
       <c r="N111" t="n">
         <v>0</v>
@@ -69022,19 +69022,19 @@
         <v>90</v>
       </c>
       <c r="K115" t="n">
-        <v>940</v>
+        <v>1005</v>
       </c>
       <c r="L115" t="n">
-        <v>629</v>
+        <v>579</v>
       </c>
       <c r="M115" t="n">
-        <v>213</v>
+        <v>148</v>
       </c>
       <c r="N115" t="n">
         <v>0</v>
       </c>
       <c r="O115" t="n">
-        <v>220</v>
+        <v>270</v>
       </c>
       <c r="P115" t="n">
         <v>4548</v>
@@ -69144,13 +69144,13 @@
         <v>302</v>
       </c>
       <c r="K117" t="n">
-        <v>910</v>
+        <v>1050</v>
       </c>
       <c r="L117" t="n">
         <v>464</v>
       </c>
       <c r="M117" t="n">
-        <v>271</v>
+        <v>131</v>
       </c>
       <c r="N117" t="n">
         <v>0</v>
@@ -69208,7 +69208,7 @@
         <v>946</v>
       </c>
       <c r="L118" t="n">
-        <v>635</v>
+        <v>550</v>
       </c>
       <c r="M118" t="n">
         <v>141</v>
@@ -69217,7 +69217,7 @@
         <v>0</v>
       </c>
       <c r="O118" t="n">
-        <v>200</v>
+        <v>285</v>
       </c>
       <c r="P118" t="n">
         <v>5746</v>
@@ -69266,13 +69266,13 @@
         <v>100</v>
       </c>
       <c r="K119" t="n">
-        <v>1364</v>
+        <v>1449</v>
       </c>
       <c r="L119" t="n">
         <v>506</v>
       </c>
       <c r="M119" t="n">
-        <v>230</v>
+        <v>145</v>
       </c>
       <c r="N119" t="n">
         <v>0</v>
@@ -69388,19 +69388,19 @@
         <v>255</v>
       </c>
       <c r="K121" t="n">
-        <v>1518</v>
+        <v>1608</v>
       </c>
       <c r="L121" t="n">
-        <v>394</v>
+        <v>354</v>
       </c>
       <c r="M121" t="n">
-        <v>236</v>
+        <v>146</v>
       </c>
       <c r="N121" t="n">
         <v>0</v>
       </c>
       <c r="O121" t="n">
-        <v>132</v>
+        <v>172</v>
       </c>
       <c r="P121" t="n">
         <v>4283</v>
@@ -69571,13 +69571,13 @@
         <v>144</v>
       </c>
       <c r="K124" t="n">
-        <v>2385</v>
+        <v>2475</v>
       </c>
       <c r="L124" t="n">
         <v>308</v>
       </c>
       <c r="M124" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="N124" t="n">
         <v>0</v>
@@ -69635,7 +69635,7 @@
         <v>549</v>
       </c>
       <c r="L125" t="n">
-        <v>429</v>
+        <v>349</v>
       </c>
       <c r="M125" t="n">
         <v>165</v>
@@ -69644,7 +69644,7 @@
         <v>0</v>
       </c>
       <c r="O125" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="P125" t="n">
         <v>4924</v>
@@ -69693,13 +69693,13 @@
         <v>0</v>
       </c>
       <c r="K126" t="n">
-        <v>1000</v>
+        <v>1120</v>
       </c>
       <c r="L126" t="n">
         <v>0</v>
       </c>
       <c r="M126" t="n">
-        <v>268</v>
+        <v>148</v>
       </c>
       <c r="N126" t="n">
         <v>0</v>
@@ -69815,19 +69815,19 @@
         <v>135</v>
       </c>
       <c r="K128" t="n">
-        <v>870</v>
+        <v>1005</v>
       </c>
       <c r="L128" t="n">
-        <v>282</v>
+        <v>237</v>
       </c>
       <c r="M128" t="n">
-        <v>264</v>
+        <v>129</v>
       </c>
       <c r="N128" t="n">
         <v>0</v>
       </c>
       <c r="O128" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="P128" t="n">
         <v>4220</v>
@@ -69998,13 +69998,13 @@
         <v>409</v>
       </c>
       <c r="K131" t="n">
-        <v>1624</v>
+        <v>1779</v>
       </c>
       <c r="L131" t="n">
         <v>240</v>
       </c>
       <c r="M131" t="n">
-        <v>304</v>
+        <v>149</v>
       </c>
       <c r="N131" t="n">
         <v>0</v>
@@ -70120,13 +70120,13 @@
         <v>0</v>
       </c>
       <c r="K133" t="n">
-        <v>1801</v>
+        <v>1921</v>
       </c>
       <c r="L133" t="n">
         <v>277</v>
       </c>
       <c r="M133" t="n">
-        <v>228</v>
+        <v>108</v>
       </c>
       <c r="N133" t="n">
         <v>0</v>
@@ -70242,13 +70242,13 @@
         <v>0</v>
       </c>
       <c r="K135" t="n">
-        <v>1710</v>
+        <v>1795</v>
       </c>
       <c r="L135" t="n">
         <v>250</v>
       </c>
       <c r="M135" t="n">
-        <v>218</v>
+        <v>133</v>
       </c>
       <c r="N135" t="n">
         <v>0</v>
@@ -70364,19 +70364,19 @@
         <v>314</v>
       </c>
       <c r="K137" t="n">
-        <v>2965</v>
+        <v>3060</v>
       </c>
       <c r="L137" t="n">
-        <v>708</v>
+        <v>558</v>
       </c>
       <c r="M137" t="n">
-        <v>254</v>
+        <v>159</v>
       </c>
       <c r="N137" t="n">
         <v>0</v>
       </c>
       <c r="O137" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="P137" t="n">
         <v>4790</v>
@@ -70529,7 +70529,7 @@
         <v>715</v>
       </c>
       <c r="E140" t="n">
-        <v>8275</v>
+        <v>9511</v>
       </c>
       <c r="F140" t="n">
         <v>7</v>
@@ -70544,16 +70544,16 @@
         <v>2635</v>
       </c>
       <c r="J140" t="n">
-        <v>0</v>
+        <v>520</v>
       </c>
       <c r="K140" t="n">
-        <v>845</v>
+        <v>2355</v>
       </c>
       <c r="L140" t="n">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="M140" t="n">
-        <v>165</v>
+        <v>0</v>
       </c>
       <c r="N140" t="n">
         <v>0</v>
@@ -70571,7 +70571,7 @@
         <v>430</v>
       </c>
       <c r="S140" t="n">
-        <v>19983</v>
+        <v>23104</v>
       </c>
     </row>
     <row r="141">
@@ -70590,7 +70590,7 @@
         <v>62862</v>
       </c>
       <c r="E141" t="n">
-        <v>863088</v>
+        <v>864324</v>
       </c>
       <c r="F141" t="n">
         <v>5937</v>
@@ -70605,22 +70605,22 @@
         <v>286740</v>
       </c>
       <c r="J141" t="n">
-        <v>4937</v>
+        <v>5457</v>
       </c>
       <c r="K141" t="n">
-        <v>109897</v>
+        <v>113789</v>
       </c>
       <c r="L141" t="n">
-        <v>35630</v>
+        <v>32932</v>
       </c>
       <c r="M141" t="n">
-        <v>8316</v>
+        <v>5769</v>
       </c>
       <c r="N141" t="n">
         <v>42</v>
       </c>
       <c r="O141" t="n">
-        <v>22098</v>
+        <v>24816</v>
       </c>
       <c r="P141" t="n">
         <v>426258</v>
@@ -70632,7 +70632,7 @@
         <v>88610</v>
       </c>
       <c r="S141" t="n">
-        <v>2089759</v>
+        <v>2092880</v>
       </c>
     </row>
   </sheetData>
@@ -76150,7 +76150,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>425</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="114">
@@ -76160,7 +76160,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>58587</v>
+        <v>59172</v>
       </c>
     </row>
     <row r="116">
@@ -76268,7 +76268,7 @@
         <v>2026</v>
       </c>
       <c r="B128" t="n">
-        <v>4530</v>
+        <v>5115</v>
       </c>
     </row>
     <row r="129">
@@ -76278,7 +76278,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>58587</v>
+        <v>59172</v>
       </c>
     </row>
   </sheetData>
@@ -77654,7 +77654,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>755</v>
+        <v>995</v>
       </c>
     </row>
     <row r="137">
@@ -77664,7 +77664,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>71327</v>
+        <v>71567</v>
       </c>
     </row>
     <row r="139">
@@ -77772,7 +77772,7 @@
         <v>2026</v>
       </c>
       <c r="B151" t="n">
-        <v>5545</v>
+        <v>5785</v>
       </c>
     </row>
     <row r="152">
@@ -77782,7 +77782,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>71327</v>
+        <v>71567</v>
       </c>
     </row>
   </sheetData>
@@ -89204,13 +89204,13 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>3435</v>
+        <v>3710</v>
       </c>
       <c r="C140" t="n">
         <v>1810</v>
       </c>
       <c r="D140" t="n">
-        <v>425</v>
+        <v>1010</v>
       </c>
       <c r="E140" t="n">
         <v>315</v>
@@ -89225,7 +89225,7 @@
         <v>0</v>
       </c>
       <c r="I140" t="n">
-        <v>7858</v>
+        <v>9879</v>
       </c>
       <c r="J140" t="n">
         <v>2490</v>
@@ -89240,13 +89240,13 @@
         <v>795</v>
       </c>
       <c r="N140" t="n">
-        <v>755</v>
+        <v>995</v>
       </c>
       <c r="O140" t="n">
         <v>220</v>
       </c>
       <c r="P140" t="n">
-        <v>19983</v>
+        <v>23104</v>
       </c>
     </row>
     <row r="141">
@@ -89256,13 +89256,13 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>400108</v>
+        <v>400383</v>
       </c>
       <c r="C141" t="n">
         <v>224962</v>
       </c>
       <c r="D141" t="n">
-        <v>58587</v>
+        <v>59172</v>
       </c>
       <c r="E141" t="n">
         <v>14604</v>
@@ -89277,7 +89277,7 @@
         <v>6860</v>
       </c>
       <c r="I141" t="n">
-        <v>756021</v>
+        <v>758042</v>
       </c>
       <c r="J141" t="n">
         <v>220401</v>
@@ -89292,13 +89292,13 @@
         <v>100763</v>
       </c>
       <c r="N141" t="n">
-        <v>71327</v>
+        <v>71567</v>
       </c>
       <c r="O141" t="n">
         <v>48837</v>
       </c>
       <c r="P141" t="n">
-        <v>2089759</v>
+        <v>2092880</v>
       </c>
     </row>
   </sheetData>
@@ -92258,7 +92258,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>3435</v>
+        <v>3710</v>
       </c>
     </row>
     <row r="141">
@@ -92268,7 +92268,7 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>400108</v>
+        <v>400383</v>
       </c>
     </row>
     <row r="143">
@@ -92376,7 +92376,7 @@
         <v>2026</v>
       </c>
       <c r="B155" t="n">
-        <v>24797</v>
+        <v>25072</v>
       </c>
     </row>
     <row r="156">
@@ -92386,7 +92386,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>400108</v>
+        <v>400383</v>
       </c>
     </row>
   </sheetData>
@@ -97215,7 +97215,7 @@
         <v>825</v>
       </c>
       <c r="M13" t="n">
-        <v>262</v>
+        <v>422</v>
       </c>
       <c r="N13" t="n">
         <v>265</v>
@@ -97230,7 +97230,7 @@
         <v>105</v>
       </c>
       <c r="R13" t="n">
-        <v>27242</v>
+        <v>27517</v>
       </c>
       <c r="S13" t="n">
         <v>190</v>
@@ -97245,7 +97245,7 @@
         <v>111</v>
       </c>
       <c r="W13" t="n">
-        <v>2370</v>
+        <v>2420</v>
       </c>
       <c r="X13" t="n">
         <v>830</v>
@@ -97290,13 +97290,13 @@
         <v>55</v>
       </c>
       <c r="AL13" t="n">
-        <v>2191</v>
+        <v>2862</v>
       </c>
       <c r="AM13" t="n">
         <v>165</v>
       </c>
       <c r="AN13" t="n">
-        <v>650</v>
+        <v>1010</v>
       </c>
       <c r="AO13" t="n">
         <v>117</v>
@@ -97308,7 +97308,7 @@
         <v>35</v>
       </c>
       <c r="AR13" t="n">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="AS13" t="n">
         <v>2140</v>
@@ -97329,7 +97329,7 @@
         <v>50</v>
       </c>
       <c r="AY13" t="n">
-        <v>2790</v>
+        <v>2870</v>
       </c>
       <c r="AZ13" t="n">
         <v>460</v>
@@ -97389,13 +97389,13 @@
         <v>1062</v>
       </c>
       <c r="BS13" t="n">
-        <v>3302</v>
+        <v>3832</v>
       </c>
       <c r="BT13" t="n">
         <v>595</v>
       </c>
       <c r="BU13" t="n">
-        <v>1035</v>
+        <v>1540</v>
       </c>
       <c r="BV13" t="n">
         <v>2727</v>
@@ -97521,7 +97521,7 @@
         <v>1825</v>
       </c>
       <c r="DK13" t="n">
-        <v>410</v>
+        <v>640</v>
       </c>
       <c r="DL13" t="n">
         <v>1903</v>
@@ -97542,7 +97542,7 @@
         <v>0</v>
       </c>
       <c r="DR13" t="n">
-        <v>5545</v>
+        <v>5785</v>
       </c>
       <c r="DS13" t="n">
         <v>275</v>
@@ -97551,7 +97551,7 @@
         <v>1730</v>
       </c>
       <c r="DU13" t="n">
-        <v>170992</v>
+        <v>174113</v>
       </c>
     </row>
     <row r="14">
@@ -97594,7 +97594,7 @@
         <v>5790</v>
       </c>
       <c r="M14" t="n">
-        <v>1582</v>
+        <v>1742</v>
       </c>
       <c r="N14" t="n">
         <v>2935</v>
@@ -97609,7 +97609,7 @@
         <v>105</v>
       </c>
       <c r="R14" t="n">
-        <v>432768</v>
+        <v>433043</v>
       </c>
       <c r="S14" t="n">
         <v>975</v>
@@ -97624,7 +97624,7 @@
         <v>14436</v>
       </c>
       <c r="W14" t="n">
-        <v>24359</v>
+        <v>24409</v>
       </c>
       <c r="X14" t="n">
         <v>4820</v>
@@ -97669,13 +97669,13 @@
         <v>427</v>
       </c>
       <c r="AL14" t="n">
-        <v>50732</v>
+        <v>51403</v>
       </c>
       <c r="AM14" t="n">
         <v>4755</v>
       </c>
       <c r="AN14" t="n">
-        <v>3355</v>
+        <v>3715</v>
       </c>
       <c r="AO14" t="n">
         <v>282</v>
@@ -97687,7 +97687,7 @@
         <v>385</v>
       </c>
       <c r="AR14" t="n">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="AS14" t="n">
         <v>26879</v>
@@ -97708,7 +97708,7 @@
         <v>460</v>
       </c>
       <c r="AY14" t="n">
-        <v>41222</v>
+        <v>41302</v>
       </c>
       <c r="AZ14" t="n">
         <v>6666</v>
@@ -97768,13 +97768,13 @@
         <v>13430</v>
       </c>
       <c r="BS14" t="n">
-        <v>26996</v>
+        <v>27526</v>
       </c>
       <c r="BT14" t="n">
         <v>5420</v>
       </c>
       <c r="BU14" t="n">
-        <v>5785</v>
+        <v>6290</v>
       </c>
       <c r="BV14" t="n">
         <v>34940</v>
@@ -97900,7 +97900,7 @@
         <v>15330</v>
       </c>
       <c r="DK14" t="n">
-        <v>10550</v>
+        <v>10780</v>
       </c>
       <c r="DL14" t="n">
         <v>18216</v>
@@ -97921,7 +97921,7 @@
         <v>1450</v>
       </c>
       <c r="DR14" t="n">
-        <v>71327</v>
+        <v>71567</v>
       </c>
       <c r="DS14" t="n">
         <v>4927</v>
@@ -97930,7 +97930,7 @@
         <v>27596</v>
       </c>
       <c r="DU14" t="n">
-        <v>2089759</v>
+        <v>2092880</v>
       </c>
     </row>
   </sheetData>
@@ -98197,7 +98197,7 @@
         <v>7433</v>
       </c>
       <c r="L4" t="n">
-        <v>3070</v>
+        <v>2795</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
@@ -98206,7 +98206,7 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>2065</v>
+        <v>2340</v>
       </c>
       <c r="P4" t="n">
         <v>30220</v>
@@ -98256,7 +98256,7 @@
         <v>7945</v>
       </c>
       <c r="L5" t="n">
-        <v>2808</v>
+        <v>2370</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -98265,7 +98265,7 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>1915</v>
+        <v>2353</v>
       </c>
       <c r="P5" t="n">
         <v>38427</v>
@@ -98315,7 +98315,7 @@
         <v>11175</v>
       </c>
       <c r="L6" t="n">
-        <v>4190</v>
+        <v>3895</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
@@ -98324,7 +98324,7 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>2115</v>
+        <v>2410</v>
       </c>
       <c r="P6" t="n">
         <v>39099</v>
@@ -98374,7 +98374,7 @@
         <v>6445</v>
       </c>
       <c r="L7" t="n">
-        <v>3210</v>
+        <v>2855</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -98383,7 +98383,7 @@
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>1455</v>
+        <v>1810</v>
       </c>
       <c r="P7" t="n">
         <v>29040</v>
@@ -98430,19 +98430,19 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>7266</v>
+        <v>7521</v>
       </c>
       <c r="L8" t="n">
-        <v>3015</v>
+        <v>2640</v>
       </c>
       <c r="M8" t="n">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
         <v>25</v>
       </c>
       <c r="O8" t="n">
-        <v>1090</v>
+        <v>1465</v>
       </c>
       <c r="P8" t="n">
         <v>35067</v>
@@ -98489,19 +98489,19 @@
         <v>94</v>
       </c>
       <c r="K9" t="n">
-        <v>9985</v>
+        <v>10425</v>
       </c>
       <c r="L9" t="n">
-        <v>3855</v>
+        <v>3500</v>
       </c>
       <c r="M9" t="n">
-        <v>1058</v>
+        <v>618</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>3273</v>
+        <v>3628</v>
       </c>
       <c r="P9" t="n">
         <v>40877</v>
@@ -98548,19 +98548,19 @@
         <v>498</v>
       </c>
       <c r="K10" t="n">
-        <v>11600</v>
+        <v>12017</v>
       </c>
       <c r="L10" t="n">
-        <v>3155</v>
+        <v>2980</v>
       </c>
       <c r="M10" t="n">
-        <v>1456</v>
+        <v>1039</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>4696</v>
+        <v>4871</v>
       </c>
       <c r="P10" t="n">
         <v>42349</v>
@@ -98607,19 +98607,19 @@
         <v>1970</v>
       </c>
       <c r="K11" t="n">
-        <v>13417</v>
+        <v>13887</v>
       </c>
       <c r="L11" t="n">
-        <v>5149</v>
+        <v>4974</v>
       </c>
       <c r="M11" t="n">
-        <v>1899</v>
+        <v>1429</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>2690</v>
+        <v>2865</v>
       </c>
       <c r="P11" t="n">
         <v>50500</v>
@@ -98666,19 +98666,19 @@
         <v>1463</v>
       </c>
       <c r="K12" t="n">
-        <v>16393</v>
+        <v>17013</v>
       </c>
       <c r="L12" t="n">
-        <v>3284</v>
+        <v>3159</v>
       </c>
       <c r="M12" t="n">
-        <v>2447</v>
+        <v>1827</v>
       </c>
       <c r="N12" t="n">
         <v>17</v>
       </c>
       <c r="O12" t="n">
-        <v>927</v>
+        <v>1052</v>
       </c>
       <c r="P12" t="n">
         <v>54184</v>
@@ -98707,7 +98707,7 @@
         <v>5550</v>
       </c>
       <c r="E13" t="n">
-        <v>71448</v>
+        <v>72684</v>
       </c>
       <c r="F13" t="n">
         <v>472</v>
@@ -98722,22 +98722,22 @@
         <v>21854</v>
       </c>
       <c r="J13" t="n">
-        <v>912</v>
+        <v>1432</v>
       </c>
       <c r="K13" t="n">
-        <v>9606</v>
+        <v>11296</v>
       </c>
       <c r="L13" t="n">
-        <v>2424</v>
+        <v>2294</v>
       </c>
       <c r="M13" t="n">
-        <v>1201</v>
+        <v>856</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>260</v>
+        <v>410</v>
       </c>
       <c r="P13" t="n">
         <v>31809</v>
@@ -98749,7 +98749,7 @@
         <v>9277</v>
       </c>
       <c r="S13" t="n">
-        <v>170992</v>
+        <v>174113</v>
       </c>
     </row>
     <row r="14">
@@ -98768,7 +98768,7 @@
         <v>62862</v>
       </c>
       <c r="E14" t="n">
-        <v>863088</v>
+        <v>864324</v>
       </c>
       <c r="F14" t="n">
         <v>5937</v>
@@ -98783,22 +98783,22 @@
         <v>286740</v>
       </c>
       <c r="J14" t="n">
-        <v>4937</v>
+        <v>5457</v>
       </c>
       <c r="K14" t="n">
-        <v>109897</v>
+        <v>113789</v>
       </c>
       <c r="L14" t="n">
-        <v>35630</v>
+        <v>32932</v>
       </c>
       <c r="M14" t="n">
-        <v>8316</v>
+        <v>5769</v>
       </c>
       <c r="N14" t="n">
         <v>42</v>
       </c>
       <c r="O14" t="n">
-        <v>22098</v>
+        <v>24816</v>
       </c>
       <c r="P14" t="n">
         <v>426258</v>
@@ -98810,7 +98810,7 @@
         <v>88610</v>
       </c>
       <c r="S14" t="n">
-        <v>2089759</v>
+        <v>2092880</v>
       </c>
     </row>
   </sheetData>
@@ -99464,13 +99464,13 @@
         <v>2026</v>
       </c>
       <c r="B13" t="n">
-        <v>24797</v>
+        <v>25072</v>
       </c>
       <c r="C13" t="n">
         <v>15989</v>
       </c>
       <c r="D13" t="n">
-        <v>4530</v>
+        <v>5115</v>
       </c>
       <c r="E13" t="n">
         <v>1955</v>
@@ -99485,7 +99485,7 @@
         <v>2690</v>
       </c>
       <c r="I13" t="n">
-        <v>73220</v>
+        <v>75241</v>
       </c>
       <c r="J13" t="n">
         <v>16330</v>
@@ -99500,13 +99500,13 @@
         <v>6260</v>
       </c>
       <c r="N13" t="n">
-        <v>5545</v>
+        <v>5785</v>
       </c>
       <c r="O13" t="n">
         <v>3865</v>
       </c>
       <c r="P13" t="n">
-        <v>170992</v>
+        <v>174113</v>
       </c>
     </row>
     <row r="14">
@@ -99516,13 +99516,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>400108</v>
+        <v>400383</v>
       </c>
       <c r="C14" t="n">
         <v>224962</v>
       </c>
       <c r="D14" t="n">
-        <v>58587</v>
+        <v>59172</v>
       </c>
       <c r="E14" t="n">
         <v>14604</v>
@@ -99537,7 +99537,7 @@
         <v>6860</v>
       </c>
       <c r="I14" t="n">
-        <v>756021</v>
+        <v>758042</v>
       </c>
       <c r="J14" t="n">
         <v>220401</v>
@@ -99552,13 +99552,13 @@
         <v>100763</v>
       </c>
       <c r="N14" t="n">
-        <v>71327</v>
+        <v>71567</v>
       </c>
       <c r="O14" t="n">
         <v>48837</v>
       </c>
       <c r="P14" t="n">
-        <v>2089759</v>
+        <v>2092880</v>
       </c>
     </row>
   </sheetData>

</xml_diff>